<commit_message>
feat: added 10 new records to restoration data
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\personal\Аспирантура\Статьи\Стаття інформ. сист\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07993584-83E5-4551-9238-4A30D4897513}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88FCAF65-7510-4B02-891A-9E8175A87192}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Лист2" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Лист1!$B$1:$H$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Лист1!$B$1:$H$27</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="552" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="612" uniqueCount="203">
   <si>
     <t>Адреса об'єкта</t>
   </si>
@@ -189,9 +189,6 @@
     <t>UA-2025-02-28-005776-a</t>
   </si>
   <si>
-    <t>м. Харків, проспект Аерокосмічний, 21</t>
-  </si>
-  <si>
     <t>UA-2025-02-14-004129-a</t>
   </si>
   <si>
@@ -321,9 +318,6 @@
     <t>UA-2023-07-28-005566-a</t>
   </si>
   <si>
-    <t>UA-2023-07-25-002621-a</t>
-  </si>
-  <si>
     <t> м. Одеса, вул. Середня, 24</t>
   </si>
   <si>
@@ -342,9 +336,6 @@
     <t>Легке</t>
   </si>
   <si>
-    <t>Чернігівська обл., с. Іванівка, вул. Шевченка, 1</t>
-  </si>
-  <si>
     <t>Оціночна площа (м²)</t>
   </si>
   <si>
@@ -498,18 +489,12 @@
     <t>вул. Центральна, 12</t>
   </si>
   <si>
-    <t>Капітальний</t>
-  </si>
-  <si>
     <t>пр. Науки, 45</t>
   </si>
   <si>
     <t>вул. Хрещатик, 22</t>
   </si>
   <si>
-    <t>Косметичний</t>
-  </si>
-  <si>
     <t>вул. Шкільна, 4</t>
   </si>
   <si>
@@ -592,6 +577,78 @@
   </si>
   <si>
     <t>вул. Гвардійська, 7</t>
+  </si>
+  <si>
+    <t>м. Запоріжжя, вул. Зестафонська, 8</t>
+  </si>
+  <si>
+    <t>UA-2024-07-03-010128-a</t>
+  </si>
+  <si>
+    <t>Реконструкція</t>
+  </si>
+  <si>
+    <t>м. Запоріжжя, вул. Зестафонська, 10</t>
+  </si>
+  <si>
+    <t>UA-2023-05-18-012968-a</t>
+  </si>
+  <si>
+    <t>м. Запоріжжя, вул. Кияшка, 22</t>
+  </si>
+  <si>
+    <t>UA-2023-05-12-010253-a</t>
+  </si>
+  <si>
+    <t>м. Запоріжжя, вул. Сталеварів, 16</t>
+  </si>
+  <si>
+    <t>UA-2023-05-23-002384-a</t>
+  </si>
+  <si>
+    <t>м. Запоріжжя, вул. Незалежної України, 80/вул. Якова Новицького, 3</t>
+  </si>
+  <si>
+    <t>UA-2023-08-01-006349-a</t>
+  </si>
+  <si>
+    <t>UA-2023-11-13-015245-a</t>
+  </si>
+  <si>
+    <t>м. Запоріжжя, вул. Сталеварів, 11</t>
+  </si>
+  <si>
+    <t>м. Запоріжжя, пр. Соборний, 151</t>
+  </si>
+  <si>
+    <t>UA-2023-08-21-012115-a</t>
+  </si>
+  <si>
+    <t>м. Дніпро, вул. Набережна Перемоги, 118</t>
+  </si>
+  <si>
+    <t>UA-2025-05-30-005516-a</t>
+  </si>
+  <si>
+    <t>м. Дніпро, вул. Енеїди, 26</t>
+  </si>
+  <si>
+    <t>UA-2024-04-17-012509-a</t>
+  </si>
+  <si>
+    <t>м. Ірпінь, вул. Шевченко, 4</t>
+  </si>
+  <si>
+    <t>UA-2023-09-22-007792-a</t>
+  </si>
+  <si>
+    <t>UA-2023-12-04-020305-a</t>
+  </si>
+  <si>
+    <t>м. Харків, пр. Льва Ландау, 27</t>
+  </si>
+  <si>
+    <t>м. Харків, пр. Аерокосмічний, 21</t>
   </si>
 </sst>
 </file>
@@ -668,7 +725,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -680,9 +737,6 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -696,6 +750,11 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Гиперссылка" xfId="1" builtinId="8"/>
@@ -977,7 +1036,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I101"/>
+  <dimension ref="A1:I111"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="50.7109375" bestFit="1" customWidth="1"/>
@@ -991,40 +1050,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
-        <v>103</v>
-      </c>
-      <c r="B1" s="9" t="s">
+      <c r="A1" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="B1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="C1" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="D1" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="E1" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="F1" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="G1" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="9" t="s">
+      <c r="H1" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="10" t="s">
-        <v>101</v>
+      <c r="I1" s="9" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="B2" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>7</v>
@@ -1038,11 +1097,11 @@
       <c r="F2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="G2" s="7">
+      <c r="G2" s="6">
         <v>32788802</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="I2">
         <v>4000</v>
@@ -1050,7 +1109,7 @@
     </row>
     <row r="3" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>29</v>
@@ -1067,7 +1126,7 @@
       <c r="F3" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="G3" s="8">
+      <c r="G3" s="7">
         <v>39493328</v>
       </c>
       <c r="H3" s="3" t="s">
@@ -1079,7 +1138,7 @@
     </row>
     <row r="4" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>28</v>
@@ -1091,12 +1150,12 @@
         <v>9</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="G4" s="8">
+      <c r="G4" s="7">
         <v>27781429</v>
       </c>
       <c r="H4" s="3" t="s">
@@ -1108,7 +1167,7 @@
     </row>
     <row r="5" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>26</v>
@@ -1125,7 +1184,7 @@
       <c r="F5" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="G5" s="8">
+      <c r="G5" s="7">
         <v>48975673</v>
       </c>
       <c r="H5" s="3" t="s">
@@ -1137,10 +1196,10 @@
     </row>
     <row r="6" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>7</v>
@@ -1154,11 +1213,11 @@
       <c r="F6" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="G6" s="8">
+      <c r="G6" s="7">
         <v>49790360</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="I6">
         <v>4000</v>
@@ -1166,7 +1225,7 @@
     </row>
     <row r="7" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>24</v>
@@ -1183,7 +1242,7 @@
       <c r="F7" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="G7" s="8">
+      <c r="G7" s="7">
         <v>63354904.399999999</v>
       </c>
       <c r="H7" s="3" t="s">
@@ -1195,10 +1254,10 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>7</v>
@@ -1212,11 +1271,11 @@
       <c r="F8" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="G8" s="8">
+      <c r="G8" s="7">
         <v>96045497</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I8">
         <v>8000</v>
@@ -1224,10 +1283,10 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>7</v>
@@ -1241,11 +1300,11 @@
       <c r="F9" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G9" s="8">
+      <c r="G9" s="7">
         <v>321652285</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="I9">
         <v>7200</v>
@@ -1253,10 +1312,10 @@
     </row>
     <row r="10" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>7</v>
@@ -1270,11 +1329,11 @@
       <c r="F10" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="G10" s="8">
+      <c r="G10" s="7">
         <v>86877046</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="I10">
         <v>3200</v>
@@ -1282,10 +1341,10 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>7</v>
@@ -1299,167 +1358,167 @@
       <c r="F11" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="G11" s="8">
+      <c r="G11" s="7">
         <v>86432499</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="I11">
         <v>4000</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>106</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D12" s="1">
+      <c r="A12" s="10" t="s">
+        <v>102</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>198</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12" s="11">
         <v>9</v>
       </c>
-      <c r="E12" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="G12" s="8">
-        <v>97455204</v>
-      </c>
-      <c r="H12" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="I12">
+      <c r="E12" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="F12" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="G12" s="12">
+        <v>57624052</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="I12" s="10">
         <v>7200</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>106</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D13" s="1">
+      <c r="A13" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>194</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D13" s="11">
         <v>9</v>
       </c>
-      <c r="E13" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="G13" s="8">
-        <v>24725271.84</v>
-      </c>
-      <c r="H13" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="I13">
+      <c r="E13" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="F13" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="G13" s="12">
+        <v>84999841</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="I13" s="10">
         <v>7200</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>106</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D14" s="1">
-        <v>5</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="G14" s="8">
-        <v>13348000</v>
-      </c>
-      <c r="H14" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="I14">
-        <v>4000</v>
+      <c r="A14" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>196</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D14" s="11">
+        <v>9</v>
+      </c>
+      <c r="E14" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="F14" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="G14" s="12">
+        <v>36595864</v>
+      </c>
+      <c r="H14" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="I14" s="10">
+        <v>7200</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>85</v>
+        <v>21</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D15" s="1">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>98</v>
+        <v>8</v>
       </c>
       <c r="F15" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="G15" s="8">
-        <v>29838682</v>
+      <c r="G15" s="7">
+        <v>97455204</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="I15">
-        <v>4000</v>
+        <v>7200</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>106</v>
-      </c>
-      <c r="B16" t="s">
-        <v>97</v>
+        <v>103</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>20</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D16" s="5">
-        <v>5</v>
+      <c r="D16" s="1">
+        <v>9</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>8</v>
+        <v>96</v>
       </c>
       <c r="F16" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="G16" s="8">
-        <v>139636363</v>
+      <c r="G16" s="7">
+        <v>24725271.84</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="I16">
-        <v>4000</v>
+        <v>7200</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>107</v>
-      </c>
-      <c r="B17" t="s">
-        <v>22</v>
+        <v>103</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>16</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>7</v>
@@ -1468,16 +1527,16 @@
         <v>5</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="F17" s="1" t="s">
         <v>15</v>
       </c>
       <c r="G17" s="7">
-        <v>15640698</v>
-      </c>
-      <c r="H17" s="4" t="s">
-        <v>96</v>
+        <v>13348000</v>
+      </c>
+      <c r="H17" s="3" t="s">
+        <v>87</v>
       </c>
       <c r="I17">
         <v>4000</v>
@@ -1485,358 +1544,358 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>108</v>
-      </c>
-      <c r="B18" t="s">
-        <v>61</v>
+        <v>103</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>84</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D18">
-        <v>12</v>
+      <c r="D18" s="1">
+        <v>5</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="F18" s="1" t="s">
         <v>15</v>
       </c>
       <c r="G18" s="7">
-        <v>50111246</v>
-      </c>
-      <c r="H18" s="4" t="s">
-        <v>62</v>
+        <v>29838682</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>85</v>
       </c>
       <c r="I18">
-        <v>9600</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>108</v>
-      </c>
-      <c r="B19" t="s">
-        <v>65</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D19">
+      <c r="A19" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="B19" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="C19" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D19" s="11">
+        <v>9</v>
+      </c>
+      <c r="E19" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="F19" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="G19" s="12">
+        <v>91668437</v>
+      </c>
+      <c r="H19" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="I19" s="10">
+        <v>7200</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="B20" s="10" t="s">
+        <v>182</v>
+      </c>
+      <c r="C20" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20" s="11">
+        <v>5</v>
+      </c>
+      <c r="E20" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="G20" s="12">
+        <v>56753765</v>
+      </c>
+      <c r="H20" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="I20" s="10">
+        <v>4000</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="B21" s="10" t="s">
+        <v>184</v>
+      </c>
+      <c r="C21" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D21" s="11">
         <v>3</v>
       </c>
-      <c r="E19" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="G19" s="7">
-        <v>14816388</v>
-      </c>
-      <c r="H19" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="I19">
+      <c r="E21" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="F21" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="G21" s="12">
+        <v>50488018</v>
+      </c>
+      <c r="H21" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="I21" s="10">
         <v>2400</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>108</v>
-      </c>
-      <c r="B20" t="s">
-        <v>67</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D20">
-        <v>9</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="G20" s="7">
-        <v>6523420</v>
-      </c>
-      <c r="H20" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="I20">
-        <v>7200</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>108</v>
-      </c>
-      <c r="B21" t="s">
-        <v>63</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D21">
-        <v>9</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="F21" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="G21" s="7">
-        <v>12815934</v>
-      </c>
-      <c r="H21" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="I21">
-        <v>7200</v>
-      </c>
-    </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>108</v>
-      </c>
-      <c r="B22" t="s">
-        <v>30</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D22">
-        <v>16</v>
-      </c>
-      <c r="E22" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F22" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="G22" s="7">
-        <v>92045720</v>
+      <c r="A22" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="B22" s="10" t="s">
+        <v>186</v>
+      </c>
+      <c r="C22" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D22" s="11">
+        <v>4</v>
+      </c>
+      <c r="E22" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="F22" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="G22" s="12">
+        <v>64471674</v>
       </c>
       <c r="H22" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="I22">
-        <v>12800</v>
+        <v>187</v>
+      </c>
+      <c r="I22" s="10">
+        <v>3200</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>108</v>
-      </c>
-      <c r="B23" t="s">
-        <v>32</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D23">
-        <v>12</v>
-      </c>
-      <c r="E23" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F23" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="G23" s="7">
-        <v>89388386</v>
+      <c r="A23" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="B23" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="C23" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D23" s="11">
+        <v>5</v>
+      </c>
+      <c r="E23" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="F23" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="G23" s="12">
+        <v>139636363</v>
       </c>
       <c r="H23" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="I23">
-        <v>9600</v>
+        <v>86</v>
+      </c>
+      <c r="I23" s="10">
+        <v>4000</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>108</v>
-      </c>
-      <c r="B24" t="s">
-        <v>35</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D24">
-        <v>12</v>
-      </c>
-      <c r="E24" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F24" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="G24" s="7">
-        <v>73774966</v>
+      <c r="A24" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="B24" s="10" t="s">
+        <v>188</v>
+      </c>
+      <c r="C24" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D24" s="11">
+        <v>5</v>
+      </c>
+      <c r="E24" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="F24" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="G24" s="12">
+        <v>214180976</v>
       </c>
       <c r="H24" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="I24">
-        <v>9600</v>
+        <v>189</v>
+      </c>
+      <c r="I24" s="10">
+        <v>4000</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>108</v>
-      </c>
-      <c r="B25" t="s">
-        <v>37</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D25">
-        <v>4</v>
-      </c>
-      <c r="E25" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F25" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="G25" s="7">
-        <v>68674967</v>
+      <c r="A25" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="B25" s="10" t="s">
+        <v>191</v>
+      </c>
+      <c r="C25" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D25" s="11">
+        <v>5</v>
+      </c>
+      <c r="E25" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="F25" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="G25" s="12">
+        <v>162165984</v>
       </c>
       <c r="H25" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="I25">
-        <v>3200</v>
+        <v>190</v>
+      </c>
+      <c r="I25" s="10">
+        <v>4000</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>108</v>
-      </c>
-      <c r="B26" t="s">
-        <v>39</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D26">
-        <v>9</v>
-      </c>
-      <c r="E26" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F26" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="G26" s="7">
-        <v>77315896</v>
+      <c r="A26" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="B26" s="10" t="s">
+        <v>192</v>
+      </c>
+      <c r="C26" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D26" s="11">
+        <v>5</v>
+      </c>
+      <c r="E26" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="F26" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="G26" s="12">
+        <v>138064624</v>
       </c>
       <c r="H26" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="I26">
-        <v>7200</v>
+        <v>193</v>
+      </c>
+      <c r="I26" s="10">
+        <v>4000</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="B27" t="s">
-        <v>41</v>
+        <v>22</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D27">
-        <v>9</v>
+      <c r="D27" s="1">
+        <v>5</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>8</v>
+        <v>97</v>
       </c>
       <c r="F27" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="G27" s="7">
-        <v>63129423</v>
+      <c r="G27" s="6">
+        <v>15640698</v>
       </c>
       <c r="H27" s="4" t="s">
-        <v>42</v>
+        <v>94</v>
       </c>
       <c r="I27">
-        <v>7200</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="B28" t="s">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="C28" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D28">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>8</v>
+        <v>96</v>
       </c>
       <c r="F28" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="G28" s="7">
-        <v>76634522</v>
+      <c r="G28" s="6">
+        <v>50111246</v>
       </c>
       <c r="H28" s="4" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="I28">
-        <v>7200</v>
+        <v>9600</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="B29" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D29">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F29" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="G29" s="7">
-        <v>32843489</v>
+      <c r="G29" s="6">
+        <v>14816388</v>
       </c>
       <c r="H29" s="4" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="I29">
-        <v>3200</v>
+        <v>2400</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="B30" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>7</v>
@@ -1845,16 +1904,16 @@
         <v>9</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="F30" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="G30" s="7">
-        <v>2948233</v>
+      <c r="G30" s="6">
+        <v>6523420</v>
       </c>
       <c r="H30" s="4" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="I30">
         <v>7200</v>
@@ -1862,132 +1921,132 @@
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="B31" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D31">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="F31" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="G31" s="7">
-        <v>22987408</v>
+      <c r="G31" s="6">
+        <v>12815934</v>
       </c>
       <c r="H31" s="4" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="I31">
-        <v>4000</v>
+        <v>7200</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>108</v>
-      </c>
-      <c r="B32" s="1" t="s">
-        <v>55</v>
+        <v>105</v>
+      </c>
+      <c r="B32" t="s">
+        <v>30</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="D32" s="1">
-        <v>2</v>
+        <v>7</v>
+      </c>
+      <c r="D32">
+        <v>16</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>98</v>
+        <v>8</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="G32" s="8">
-        <v>2972856</v>
-      </c>
-      <c r="H32" s="3" t="s">
-        <v>57</v>
+        <v>15</v>
+      </c>
+      <c r="G32" s="6">
+        <v>92045720</v>
+      </c>
+      <c r="H32" s="4" t="s">
+        <v>31</v>
       </c>
       <c r="I32">
-        <v>1600</v>
+        <v>12800</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>108</v>
-      </c>
-      <c r="B33" s="1" t="s">
-        <v>58</v>
+        <v>105</v>
+      </c>
+      <c r="B33" t="s">
+        <v>32</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="D33" s="1">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="D33">
+        <v>12</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>98</v>
+        <v>8</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="G33" s="8">
-        <v>27299654.399999999</v>
-      </c>
-      <c r="H33" s="3" t="s">
-        <v>60</v>
+        <v>15</v>
+      </c>
+      <c r="G33" s="6">
+        <v>89388386</v>
+      </c>
+      <c r="H33" s="4" t="s">
+        <v>33</v>
       </c>
       <c r="I33">
-        <v>4800</v>
+        <v>9600</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>108</v>
-      </c>
-      <c r="B34" s="1" t="s">
-        <v>46</v>
+        <v>105</v>
+      </c>
+      <c r="B34" t="s">
+        <v>35</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D34" s="1">
-        <v>5</v>
+      <c r="D34">
+        <v>12</v>
       </c>
       <c r="E34" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="G34" s="8">
-        <v>16999485</v>
-      </c>
-      <c r="H34" s="3" t="s">
-        <v>10</v>
+        <v>15</v>
+      </c>
+      <c r="G34" s="6">
+        <v>73774966</v>
+      </c>
+      <c r="H34" s="4" t="s">
+        <v>36</v>
       </c>
       <c r="I34">
-        <v>4000</v>
+        <v>9600</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>108</v>
-      </c>
-      <c r="B35" s="1" t="s">
-        <v>47</v>
+        <v>105</v>
+      </c>
+      <c r="B35" t="s">
+        <v>37</v>
       </c>
       <c r="C35" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D35" s="1">
-        <v>9</v>
+      <c r="D35">
+        <v>4</v>
       </c>
       <c r="E35" s="1" t="s">
         <v>8</v>
@@ -1995,85 +2054,85 @@
       <c r="F35" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="G35" s="8">
-        <v>44441057</v>
-      </c>
-      <c r="H35" s="3" t="s">
-        <v>48</v>
+      <c r="G35" s="6">
+        <v>68674967</v>
+      </c>
+      <c r="H35" s="4" t="s">
+        <v>38</v>
       </c>
       <c r="I35">
-        <v>7200</v>
+        <v>3200</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>108</v>
-      </c>
-      <c r="B36" s="1" t="s">
-        <v>13</v>
+        <v>105</v>
+      </c>
+      <c r="B36" t="s">
+        <v>39</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D36" s="1">
-        <v>4</v>
+        <v>7</v>
+      </c>
+      <c r="D36">
+        <v>9</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>98</v>
+        <v>8</v>
       </c>
       <c r="F36" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="G36" s="8">
-        <v>25943436</v>
-      </c>
-      <c r="H36" s="3" t="s">
-        <v>45</v>
+      <c r="G36" s="6">
+        <v>77315896</v>
+      </c>
+      <c r="H36" s="4" t="s">
+        <v>40</v>
       </c>
       <c r="I36">
-        <v>3200</v>
+        <v>7200</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="B37" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D37">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>98</v>
+        <v>8</v>
       </c>
       <c r="F37" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="G37" s="7">
-        <v>13930986</v>
+      <c r="G37" s="6">
+        <v>63129423</v>
       </c>
       <c r="H37" s="4" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="I37">
-        <v>4000</v>
+        <v>7200</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>110</v>
-      </c>
-      <c r="B38" s="1" t="s">
-        <v>34</v>
+        <v>105</v>
+      </c>
+      <c r="B38" t="s">
+        <v>50</v>
       </c>
       <c r="C38" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D38" s="1">
+      <c r="D38">
         <v>9</v>
       </c>
       <c r="E38" s="1" t="s">
@@ -2082,11 +2141,11 @@
       <c r="F38" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="G38" s="8">
-        <v>45955000</v>
-      </c>
-      <c r="H38" s="3" t="s">
-        <v>23</v>
+      <c r="G38" s="6">
+        <v>76634522</v>
+      </c>
+      <c r="H38" s="4" t="s">
+        <v>51</v>
       </c>
       <c r="I38">
         <v>7200</v>
@@ -2094,285 +2153,306 @@
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="B39" t="s">
-        <v>89</v>
+        <v>70</v>
       </c>
       <c r="C39" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D39">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>8</v>
+        <v>96</v>
       </c>
       <c r="F39" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="G39" s="7">
-        <v>44103000</v>
+      <c r="G39" s="6">
+        <v>32843489</v>
       </c>
       <c r="H39" s="4" t="s">
-        <v>90</v>
+        <v>71</v>
       </c>
       <c r="I39">
-        <v>4000</v>
+        <v>3200</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="B40" t="s">
-        <v>91</v>
+        <v>68</v>
       </c>
       <c r="C40" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D40">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F40" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="G40" s="7">
-        <v>26576000</v>
+      <c r="G40" s="6">
+        <v>2948233</v>
       </c>
       <c r="H40" s="4" t="s">
-        <v>92</v>
+        <v>69</v>
       </c>
       <c r="I40">
-        <v>4000</v>
+        <v>7200</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="B41" t="s">
-        <v>100</v>
+        <v>52</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="D41">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="F41" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="G41" s="7">
-        <v>14462000</v>
+      <c r="G41" s="6">
+        <v>22987408</v>
       </c>
       <c r="H41" s="4" t="s">
-        <v>93</v>
+        <v>53</v>
       </c>
       <c r="I41">
-        <v>800</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>108</v>
-      </c>
-      <c r="B42" t="s">
-        <v>102</v>
-      </c>
-      <c r="C42" t="s">
-        <v>7</v>
-      </c>
-      <c r="D42">
-        <v>9</v>
-      </c>
-      <c r="E42" t="s">
-        <v>8</v>
-      </c>
-      <c r="F42" t="s">
-        <v>15</v>
+        <v>105</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D42" s="1">
+        <v>2</v>
+      </c>
+      <c r="E42" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F42" s="1" t="s">
+        <v>55</v>
       </c>
       <c r="G42" s="7">
-        <v>82500000</v>
+        <v>2972856</v>
+      </c>
+      <c r="H42" s="3" t="s">
+        <v>56</v>
       </c>
       <c r="I42">
-        <v>7425</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>108</v>
-      </c>
-      <c r="B43" t="s">
-        <v>114</v>
-      </c>
-      <c r="C43" t="s">
-        <v>7</v>
-      </c>
-      <c r="D43">
-        <v>5</v>
-      </c>
-      <c r="E43" t="s">
-        <v>98</v>
-      </c>
-      <c r="F43" t="s">
-        <v>15</v>
+        <v>105</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D43" s="1">
+        <v>6</v>
+      </c>
+      <c r="E43" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F43" s="1" t="s">
+        <v>55</v>
       </c>
       <c r="G43" s="7">
-        <v>37200000</v>
+        <v>27299654.399999999</v>
+      </c>
+      <c r="H43" s="3" t="s">
+        <v>59</v>
       </c>
       <c r="I43">
-        <v>3720</v>
+        <v>4800</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>107</v>
-      </c>
-      <c r="B44" t="s">
-        <v>115</v>
-      </c>
-      <c r="C44" t="s">
-        <v>7</v>
-      </c>
-      <c r="D44">
+        <v>105</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D44" s="1">
+        <v>5</v>
+      </c>
+      <c r="E44" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F44" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E44" t="s">
-        <v>98</v>
-      </c>
-      <c r="F44" t="s">
-        <v>15</v>
-      </c>
       <c r="G44" s="7">
-        <v>45000000</v>
+        <v>16999485</v>
+      </c>
+      <c r="H44" s="3" t="s">
+        <v>10</v>
       </c>
       <c r="I44">
-        <v>4500</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>104</v>
-      </c>
-      <c r="B45" t="s">
-        <v>116</v>
-      </c>
-      <c r="C45" t="s">
-        <v>7</v>
-      </c>
-      <c r="D45">
-        <v>5</v>
-      </c>
-      <c r="E45" t="s">
-        <v>99</v>
-      </c>
-      <c r="F45" t="s">
+        <v>105</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D45" s="1">
+        <v>9</v>
+      </c>
+      <c r="E45" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F45" s="1" t="s">
         <v>15</v>
       </c>
       <c r="G45" s="7">
-        <v>21800000</v>
+        <v>44441057</v>
+      </c>
+      <c r="H45" s="3" t="s">
+        <v>48</v>
       </c>
       <c r="I45">
-        <v>2180</v>
+        <v>7200</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>123</v>
-      </c>
-      <c r="B46" t="s">
-        <v>117</v>
-      </c>
-      <c r="C46" t="s">
-        <v>7</v>
-      </c>
-      <c r="D46">
+        <v>105</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D46" s="1">
         <v>4</v>
       </c>
-      <c r="E46" t="s">
-        <v>98</v>
-      </c>
-      <c r="F46" t="s">
+      <c r="E46" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F46" s="1" t="s">
         <v>15</v>
       </c>
       <c r="G46" s="7">
-        <v>28900000</v>
+        <v>25943436</v>
+      </c>
+      <c r="H46" s="3" t="s">
+        <v>45</v>
       </c>
       <c r="I46">
-        <v>2890</v>
+        <v>3200</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="B47" t="s">
-        <v>118</v>
-      </c>
-      <c r="C47" t="s">
+        <v>202</v>
+      </c>
+      <c r="C47" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D47">
-        <v>9</v>
-      </c>
-      <c r="E47" t="s">
-        <v>8</v>
-      </c>
-      <c r="F47" t="s">
-        <v>15</v>
-      </c>
-      <c r="G47" s="7">
-        <v>74100000</v>
+        <v>5</v>
+      </c>
+      <c r="E47" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F47" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G47" s="6">
+        <v>13930986</v>
+      </c>
+      <c r="H47" s="4" t="s">
+        <v>49</v>
       </c>
       <c r="I47">
-        <v>7410</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
+      <c r="A48" s="10" t="s">
         <v>105</v>
       </c>
-      <c r="B48" t="s">
-        <v>119</v>
-      </c>
-      <c r="C48" t="s">
-        <v>7</v>
-      </c>
-      <c r="D48">
-        <v>12</v>
-      </c>
-      <c r="E48" t="s">
-        <v>8</v>
-      </c>
-      <c r="F48" t="s">
-        <v>15</v>
-      </c>
-      <c r="G48" s="7">
-        <v>97000000</v>
-      </c>
-      <c r="I48">
-        <v>9600</v>
+      <c r="B48" s="10" t="s">
+        <v>201</v>
+      </c>
+      <c r="C48" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="D48" s="10">
+        <v>4</v>
+      </c>
+      <c r="E48" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="F48" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="G48" s="12">
+        <v>60558384</v>
+      </c>
+      <c r="H48" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="I48" s="10">
+        <v>3200</v>
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>105</v>
-      </c>
-      <c r="B49" t="s">
-        <v>120</v>
+        <v>107</v>
+      </c>
+      <c r="B49" s="1" t="s">
+        <v>34</v>
       </c>
       <c r="C49" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D49" s="1">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E49" s="1" t="s">
         <v>8</v>
@@ -2380,555 +2460,564 @@
       <c r="F49" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="G49" s="8">
-        <v>39800000</v>
-      </c>
-      <c r="H49" s="1"/>
-      <c r="I49" s="6">
-        <v>3980</v>
+      <c r="G49" s="7">
+        <v>45955000</v>
+      </c>
+      <c r="H49" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="I49">
+        <v>7200</v>
       </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>124</v>
+        <v>108</v>
       </c>
       <c r="B50" t="s">
-        <v>122</v>
+        <v>88</v>
       </c>
       <c r="C50" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D50" s="1">
-        <v>9</v>
+      <c r="D50">
+        <v>5</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>98</v>
+        <v>8</v>
       </c>
       <c r="F50" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="G50" s="8">
-        <v>44000000</v>
-      </c>
-      <c r="H50" s="1"/>
-      <c r="I50" s="6">
-        <v>4400</v>
+      <c r="G50" s="6">
+        <v>44103000</v>
+      </c>
+      <c r="H50" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="I50">
+        <v>4000</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>125</v>
+        <v>108</v>
       </c>
       <c r="B51" t="s">
-        <v>121</v>
+        <v>90</v>
       </c>
       <c r="C51" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D51" s="1">
+      <c r="D51">
         <v>5</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="F51" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="G51" s="8">
-        <v>31000000</v>
-      </c>
-      <c r="H51" s="1"/>
-      <c r="I51" s="6">
-        <v>3100</v>
+      <c r="G51" s="6">
+        <v>26576000</v>
+      </c>
+      <c r="H51" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="I51">
+        <v>4000</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A52" s="1" t="s">
-        <v>146</v>
+      <c r="A52" t="s">
+        <v>105</v>
       </c>
       <c r="B52" t="s">
-        <v>126</v>
-      </c>
-      <c r="C52" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D52" s="1">
+        <v>99</v>
+      </c>
+      <c r="C52" t="s">
+        <v>7</v>
+      </c>
+      <c r="D52">
         <v>9</v>
       </c>
-      <c r="E52" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="F52" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="G52" s="8">
-        <v>42000000</v>
-      </c>
-      <c r="H52" s="2"/>
+      <c r="E52" t="s">
+        <v>8</v>
+      </c>
+      <c r="F52" t="s">
+        <v>15</v>
+      </c>
+      <c r="G52" s="6">
+        <v>82500000</v>
+      </c>
       <c r="I52">
         <v>7425</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A53" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="B53" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="C53" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D53" s="1">
+      <c r="A53" t="s">
+        <v>105</v>
+      </c>
+      <c r="B53" t="s">
+        <v>111</v>
+      </c>
+      <c r="C53" t="s">
+        <v>7</v>
+      </c>
+      <c r="D53">
         <v>5</v>
       </c>
-      <c r="E53" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F53" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="G53" s="8">
-        <v>39600000</v>
-      </c>
-      <c r="H53" s="2"/>
+      <c r="E53" t="s">
+        <v>96</v>
+      </c>
+      <c r="F53" t="s">
+        <v>15</v>
+      </c>
+      <c r="G53" s="6">
+        <v>37200000</v>
+      </c>
       <c r="I53">
-        <v>4125</v>
+        <v>3720</v>
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A54" s="1" t="s">
+      <c r="A54" t="s">
+        <v>104</v>
+      </c>
+      <c r="B54" t="s">
+        <v>112</v>
+      </c>
+      <c r="C54" t="s">
+        <v>7</v>
+      </c>
+      <c r="D54">
+        <v>9</v>
+      </c>
+      <c r="E54" t="s">
+        <v>96</v>
+      </c>
+      <c r="F54" t="s">
+        <v>15</v>
+      </c>
+      <c r="G54" s="6">
+        <v>45000000</v>
+      </c>
+      <c r="I54">
+        <v>4500</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>101</v>
+      </c>
+      <c r="B55" t="s">
         <v>113</v>
       </c>
-      <c r="B54" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="C54" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D54" s="1">
+      <c r="C55" t="s">
+        <v>7</v>
+      </c>
+      <c r="D55">
+        <v>5</v>
+      </c>
+      <c r="E55" t="s">
+        <v>97</v>
+      </c>
+      <c r="F55" t="s">
+        <v>15</v>
+      </c>
+      <c r="G55" s="6">
+        <v>21800000</v>
+      </c>
+      <c r="I55">
+        <v>2180</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>120</v>
+      </c>
+      <c r="B56" t="s">
+        <v>114</v>
+      </c>
+      <c r="C56" t="s">
+        <v>7</v>
+      </c>
+      <c r="D56">
+        <v>4</v>
+      </c>
+      <c r="E56" t="s">
+        <v>96</v>
+      </c>
+      <c r="F56" t="s">
+        <v>15</v>
+      </c>
+      <c r="G56" s="6">
+        <v>28900000</v>
+      </c>
+      <c r="I56">
+        <v>2890</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>110</v>
+      </c>
+      <c r="B57" t="s">
+        <v>115</v>
+      </c>
+      <c r="C57" t="s">
+        <v>7</v>
+      </c>
+      <c r="D57">
         <v>9</v>
       </c>
-      <c r="E54" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="F54" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="G54" s="8">
-        <v>40800000</v>
-      </c>
-      <c r="H54" s="2"/>
-      <c r="I54">
-        <v>7425</v>
-      </c>
-    </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A55" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="B55" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="C55" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D55" s="1">
-        <v>4</v>
-      </c>
-      <c r="E55" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="F55" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="G55" s="8">
-        <v>29300000</v>
-      </c>
-      <c r="H55" s="2"/>
-      <c r="I55">
-        <v>3300</v>
-      </c>
-    </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A56" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="B56" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="C56" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D56" s="1">
+      <c r="E57" t="s">
+        <v>8</v>
+      </c>
+      <c r="F57" t="s">
+        <v>15</v>
+      </c>
+      <c r="G57" s="6">
+        <v>74100000</v>
+      </c>
+      <c r="I57">
+        <v>7410</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>102</v>
+      </c>
+      <c r="B58" t="s">
+        <v>116</v>
+      </c>
+      <c r="C58" t="s">
+        <v>7</v>
+      </c>
+      <c r="D58">
+        <v>12</v>
+      </c>
+      <c r="E58" t="s">
+        <v>8</v>
+      </c>
+      <c r="F58" t="s">
+        <v>15</v>
+      </c>
+      <c r="G58" s="6">
+        <v>97000000</v>
+      </c>
+      <c r="I58">
+        <v>9600</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>102</v>
+      </c>
+      <c r="B59" t="s">
+        <v>117</v>
+      </c>
+      <c r="C59" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D59" s="1">
         <v>5</v>
       </c>
-      <c r="E56" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="F56" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="G56" s="8">
-        <v>19200000</v>
-      </c>
-      <c r="H56" s="2"/>
-      <c r="I56">
-        <v>4125</v>
-      </c>
-    </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A57" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="B57" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="C57" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D57" s="1">
-        <v>12</v>
-      </c>
-      <c r="E57" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F57" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="G57" s="8">
-        <v>87100000</v>
-      </c>
-      <c r="H57" s="2"/>
-      <c r="I57">
-        <v>9900</v>
-      </c>
-    </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A58" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="B58" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="C58" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D58" s="1">
+      <c r="E59" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F59" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G59" s="7">
+        <v>39800000</v>
+      </c>
+      <c r="H59" s="1"/>
+      <c r="I59" s="5">
+        <v>3980</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>121</v>
+      </c>
+      <c r="B60" t="s">
+        <v>119</v>
+      </c>
+      <c r="C60" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D60" s="1">
         <v>9</v>
       </c>
-      <c r="E58" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F58" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="G58" s="8">
-        <v>75200000</v>
-      </c>
-      <c r="H58" s="2"/>
-      <c r="I58">
-        <v>7425</v>
-      </c>
-    </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A59" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="B59" t="s">
-        <v>133</v>
-      </c>
-      <c r="C59" t="s">
-        <v>7</v>
-      </c>
-      <c r="D59">
-        <v>5</v>
-      </c>
-      <c r="E59" t="s">
-        <v>98</v>
-      </c>
-      <c r="F59" t="s">
-        <v>15</v>
-      </c>
-      <c r="G59" s="7">
-        <v>36700000</v>
-      </c>
-      <c r="I59">
-        <v>4125</v>
-      </c>
-    </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A60" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="B60" t="s">
-        <v>134</v>
-      </c>
-      <c r="C60" t="s">
-        <v>7</v>
-      </c>
-      <c r="D60">
-        <v>5</v>
-      </c>
-      <c r="E60" t="s">
-        <v>8</v>
-      </c>
-      <c r="F60" t="s">
+      <c r="E60" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F60" s="1" t="s">
         <v>15</v>
       </c>
       <c r="G60" s="7">
-        <v>40000000</v>
-      </c>
-      <c r="I60">
-        <v>4125</v>
+        <v>44000000</v>
+      </c>
+      <c r="H60" s="1"/>
+      <c r="I60" s="5">
+        <v>4400</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>105</v>
+        <v>122</v>
       </c>
       <c r="B61" t="s">
-        <v>135</v>
-      </c>
-      <c r="C61" t="s">
-        <v>7</v>
-      </c>
-      <c r="D61">
-        <v>10</v>
-      </c>
-      <c r="E61" t="s">
-        <v>8</v>
-      </c>
-      <c r="F61" t="s">
+        <v>118</v>
+      </c>
+      <c r="C61" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D61" s="1">
+        <v>5</v>
+      </c>
+      <c r="E61" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F61" s="1" t="s">
         <v>15</v>
       </c>
       <c r="G61" s="7">
-        <v>91000000</v>
-      </c>
-      <c r="I61">
-        <v>8250</v>
+        <v>31000000</v>
+      </c>
+      <c r="H61" s="1"/>
+      <c r="I61" s="5">
+        <v>3100</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A62" t="s">
-        <v>146</v>
+      <c r="A62" s="1" t="s">
+        <v>143</v>
       </c>
       <c r="B62" t="s">
-        <v>136</v>
-      </c>
-      <c r="C62" t="s">
-        <v>7</v>
-      </c>
-      <c r="D62">
+        <v>123</v>
+      </c>
+      <c r="C62" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D62" s="1">
         <v>9</v>
       </c>
-      <c r="E62" t="s">
-        <v>99</v>
-      </c>
-      <c r="F62" t="s">
+      <c r="E62" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F62" s="1" t="s">
         <v>15</v>
       </c>
       <c r="G62" s="7">
-        <v>28600000</v>
-      </c>
+        <v>42000000</v>
+      </c>
+      <c r="H62" s="2"/>
       <c r="I62">
         <v>7425</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A63" t="s">
-        <v>125</v>
-      </c>
-      <c r="B63" t="s">
-        <v>137</v>
-      </c>
-      <c r="C63" t="s">
-        <v>7</v>
-      </c>
-      <c r="D63">
+      <c r="A63" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="B63" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="C63" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D63" s="1">
         <v>5</v>
       </c>
-      <c r="E63" t="s">
-        <v>98</v>
-      </c>
-      <c r="F63" t="s">
+      <c r="E63" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F63" s="1" t="s">
         <v>15</v>
       </c>
       <c r="G63" s="7">
-        <v>34400000</v>
-      </c>
+        <v>39600000</v>
+      </c>
+      <c r="H63" s="2"/>
       <c r="I63">
         <v>4125</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A64" t="s">
-        <v>147</v>
-      </c>
-      <c r="B64" t="s">
-        <v>138</v>
-      </c>
-      <c r="C64" t="s">
-        <v>7</v>
-      </c>
-      <c r="D64">
+      <c r="A64" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="B64" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C64" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D64" s="1">
         <v>9</v>
       </c>
-      <c r="E64" t="s">
-        <v>8</v>
-      </c>
-      <c r="F64" t="s">
+      <c r="E64" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F64" s="1" t="s">
         <v>15</v>
       </c>
       <c r="G64" s="7">
-        <v>65800000</v>
-      </c>
+        <v>40800000</v>
+      </c>
+      <c r="H64" s="2"/>
       <c r="I64">
         <v>7425</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A65" t="s">
-        <v>105</v>
-      </c>
-      <c r="B65" t="s">
-        <v>139</v>
-      </c>
-      <c r="C65" t="s">
-        <v>7</v>
-      </c>
-      <c r="D65">
+      <c r="A65" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B65" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="C65" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D65" s="1">
+        <v>4</v>
+      </c>
+      <c r="E65" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F65" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G65" s="7">
+        <v>29300000</v>
+      </c>
+      <c r="H65" s="2"/>
+      <c r="I65">
+        <v>3300</v>
+      </c>
+    </row>
+    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A66" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B66" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="C66" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D66" s="1">
         <v>5</v>
       </c>
-      <c r="E65" t="s">
-        <v>8</v>
-      </c>
-      <c r="F65" t="s">
-        <v>15</v>
-      </c>
-      <c r="G65" s="7">
-        <v>47000000</v>
-      </c>
-      <c r="I65">
-        <v>4125</v>
-      </c>
-    </row>
-    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A66" t="s">
-        <v>105</v>
-      </c>
-      <c r="B66" t="s">
-        <v>140</v>
-      </c>
-      <c r="C66" t="s">
-        <v>7</v>
-      </c>
-      <c r="D66">
-        <v>5</v>
-      </c>
-      <c r="E66" t="s">
-        <v>98</v>
-      </c>
-      <c r="F66" t="s">
+      <c r="E66" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="F66" s="1" t="s">
         <v>15</v>
       </c>
       <c r="G66" s="7">
-        <v>30900000</v>
-      </c>
+        <v>19200000</v>
+      </c>
+      <c r="H66" s="2"/>
       <c r="I66">
         <v>4125</v>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A67" t="s">
-        <v>124</v>
-      </c>
-      <c r="B67" t="s">
-        <v>141</v>
-      </c>
-      <c r="C67" t="s">
-        <v>7</v>
-      </c>
-      <c r="D67">
+      <c r="A67" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="B67" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="C67" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D67" s="1">
+        <v>12</v>
+      </c>
+      <c r="E67" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F67" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G67" s="7">
+        <v>87100000</v>
+      </c>
+      <c r="H67" s="2"/>
+      <c r="I67">
+        <v>9900</v>
+      </c>
+    </row>
+    <row r="68" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A68" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="C68" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D68" s="1">
         <v>9</v>
       </c>
-      <c r="E67" t="s">
-        <v>98</v>
-      </c>
-      <c r="F67" t="s">
-        <v>15</v>
-      </c>
-      <c r="G67" s="7">
-        <v>41200000</v>
-      </c>
-      <c r="I67">
+      <c r="E68" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F68" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G68" s="7">
+        <v>75200000</v>
+      </c>
+      <c r="H68" s="2"/>
+      <c r="I68">
         <v>7425</v>
       </c>
     </row>
-    <row r="68" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A68" t="s">
-        <v>123</v>
-      </c>
-      <c r="B68" t="s">
-        <v>142</v>
-      </c>
-      <c r="C68" t="s">
-        <v>7</v>
-      </c>
-      <c r="D68">
+    <row r="69" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A69" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="B69" t="s">
+        <v>130</v>
+      </c>
+      <c r="C69" t="s">
+        <v>7</v>
+      </c>
+      <c r="D69">
         <v>5</v>
       </c>
-      <c r="E68" t="s">
-        <v>8</v>
-      </c>
-      <c r="F68" t="s">
-        <v>15</v>
-      </c>
-      <c r="G68" s="7">
-        <v>38500000</v>
-      </c>
-      <c r="I68">
+      <c r="E69" t="s">
+        <v>96</v>
+      </c>
+      <c r="F69" t="s">
+        <v>15</v>
+      </c>
+      <c r="G69" s="6">
+        <v>36700000</v>
+      </c>
+      <c r="I69">
         <v>4125</v>
       </c>
     </row>
-    <row r="69" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A69" t="s">
-        <v>149</v>
-      </c>
-      <c r="B69" t="s">
-        <v>143</v>
-      </c>
-      <c r="C69" t="s">
-        <v>7</v>
-      </c>
-      <c r="D69">
-        <v>4</v>
-      </c>
-      <c r="E69" t="s">
-        <v>98</v>
-      </c>
-      <c r="F69" t="s">
-        <v>15</v>
-      </c>
-      <c r="G69" s="7">
-        <v>25700000</v>
-      </c>
-      <c r="I69">
-        <v>3300</v>
-      </c>
-    </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A70" t="s">
-        <v>108</v>
+      <c r="A70" s="1" t="s">
+        <v>145</v>
       </c>
       <c r="B70" t="s">
-        <v>144</v>
+        <v>131</v>
       </c>
       <c r="C70" t="s">
         <v>7</v>
       </c>
       <c r="D70">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="E70" t="s">
         <v>8</v>
@@ -2936,643 +3025,643 @@
       <c r="F70" t="s">
         <v>15</v>
       </c>
-      <c r="G70" s="7">
-        <v>80400000</v>
+      <c r="G70" s="6">
+        <v>40000000</v>
       </c>
       <c r="I70">
-        <v>7425</v>
+        <v>4125</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A71" s="1" t="s">
-        <v>148</v>
+      <c r="A71" t="s">
+        <v>102</v>
       </c>
       <c r="B71" t="s">
-        <v>145</v>
+        <v>132</v>
       </c>
       <c r="C71" t="s">
         <v>7</v>
       </c>
       <c r="D71">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E71" t="s">
-        <v>99</v>
+        <v>8</v>
       </c>
       <c r="F71" t="s">
         <v>15</v>
       </c>
-      <c r="G71" s="7">
-        <v>21300000</v>
+      <c r="G71" s="6">
+        <v>91000000</v>
       </c>
       <c r="I71">
-        <v>4125</v>
+        <v>8250</v>
       </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>150</v>
+        <v>143</v>
       </c>
       <c r="B72" t="s">
-        <v>151</v>
+        <v>133</v>
       </c>
       <c r="C72" t="s">
         <v>7</v>
       </c>
       <c r="D72">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E72" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F72" t="s">
-        <v>152</v>
-      </c>
-      <c r="G72">
-        <v>20800000</v>
+        <v>15</v>
+      </c>
+      <c r="G72" s="6">
+        <v>28600000</v>
       </c>
       <c r="I72">
-        <v>4000</v>
+        <v>7425</v>
       </c>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>108</v>
+        <v>122</v>
       </c>
       <c r="B73" t="s">
-        <v>153</v>
+        <v>134</v>
       </c>
       <c r="C73" t="s">
         <v>7</v>
       </c>
       <c r="D73">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="E73" t="s">
-        <v>8</v>
+        <v>96</v>
       </c>
       <c r="F73" t="s">
-        <v>152</v>
-      </c>
-      <c r="G73">
-        <v>64800000</v>
+        <v>15</v>
+      </c>
+      <c r="G73" s="6">
+        <v>34400000</v>
       </c>
       <c r="I73">
-        <v>7200</v>
+        <v>4125</v>
       </c>
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="B74" t="s">
-        <v>154</v>
+        <v>135</v>
       </c>
       <c r="C74" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="D74">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E74" t="s">
-        <v>99</v>
+        <v>8</v>
       </c>
       <c r="F74" t="s">
-        <v>155</v>
-      </c>
-      <c r="G74">
-        <v>10560000</v>
+        <v>15</v>
+      </c>
+      <c r="G74" s="6">
+        <v>65800000</v>
       </c>
       <c r="I74">
-        <v>3200</v>
+        <v>7425</v>
       </c>
     </row>
     <row r="75" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="B75" t="s">
-        <v>156</v>
+        <v>136</v>
       </c>
       <c r="C75" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="D75">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E75" t="s">
-        <v>98</v>
+        <v>8</v>
       </c>
       <c r="F75" t="s">
-        <v>152</v>
-      </c>
-      <c r="G75">
-        <v>3520000</v>
+        <v>15</v>
+      </c>
+      <c r="G75" s="6">
+        <v>47000000</v>
       </c>
       <c r="I75">
-        <v>800</v>
+        <v>4125</v>
       </c>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B76" t="s">
-        <v>157</v>
+        <v>137</v>
       </c>
       <c r="C76" t="s">
         <v>7</v>
       </c>
       <c r="D76">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E76" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="F76" t="s">
-        <v>155</v>
-      </c>
-      <c r="G76">
-        <v>7560000</v>
+        <v>15</v>
+      </c>
+      <c r="G76" s="6">
+        <v>30900000</v>
       </c>
       <c r="I76">
-        <v>2400</v>
+        <v>4125</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>107</v>
+        <v>121</v>
       </c>
       <c r="B77" t="s">
-        <v>158</v>
+        <v>138</v>
       </c>
       <c r="C77" t="s">
         <v>7</v>
       </c>
       <c r="D77">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E77" t="s">
-        <v>8</v>
+        <v>96</v>
       </c>
       <c r="F77" t="s">
-        <v>152</v>
-      </c>
-      <c r="G77">
-        <v>91200000</v>
+        <v>15</v>
+      </c>
+      <c r="G77" s="6">
+        <v>41200000</v>
       </c>
       <c r="I77">
-        <v>9600</v>
+        <v>7425</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>159</v>
+        <v>120</v>
       </c>
       <c r="B78" t="s">
-        <v>160</v>
+        <v>139</v>
       </c>
       <c r="C78" t="s">
-        <v>59</v>
+        <v>7</v>
       </c>
       <c r="D78">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E78" t="s">
-        <v>98</v>
+        <v>8</v>
       </c>
       <c r="F78" t="s">
-        <v>152</v>
-      </c>
-      <c r="G78">
-        <v>28800000</v>
+        <v>15</v>
+      </c>
+      <c r="G78" s="6">
+        <v>38500000</v>
       </c>
       <c r="I78">
-        <v>4800</v>
+        <v>4125</v>
       </c>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>159</v>
+        <v>146</v>
       </c>
       <c r="B79" t="s">
-        <v>161</v>
+        <v>140</v>
       </c>
       <c r="C79" t="s">
-        <v>59</v>
+        <v>7</v>
       </c>
       <c r="D79">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E79" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="F79" t="s">
-        <v>152</v>
-      </c>
-      <c r="G79">
-        <v>9600000</v>
+        <v>15</v>
+      </c>
+      <c r="G79" s="6">
+        <v>25700000</v>
       </c>
       <c r="I79">
-        <v>1600</v>
+        <v>3300</v>
       </c>
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="B80" t="s">
-        <v>162</v>
+        <v>141</v>
       </c>
       <c r="C80" t="s">
         <v>7</v>
       </c>
       <c r="D80">
+        <v>9</v>
+      </c>
+      <c r="E80" t="s">
+        <v>8</v>
+      </c>
+      <c r="F80" t="s">
+        <v>15</v>
+      </c>
+      <c r="G80" s="6">
+        <v>80400000</v>
+      </c>
+      <c r="I80">
+        <v>7425</v>
+      </c>
+    </row>
+    <row r="81" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A81" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="B81" t="s">
+        <v>142</v>
+      </c>
+      <c r="C81" t="s">
+        <v>7</v>
+      </c>
+      <c r="D81">
         <v>5</v>
       </c>
-      <c r="E80" t="s">
-        <v>98</v>
-      </c>
-      <c r="F80" t="s">
-        <v>152</v>
-      </c>
-      <c r="G80">
-        <v>20800000</v>
-      </c>
-      <c r="I80">
-        <v>4000</v>
-      </c>
-    </row>
-    <row r="81" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A81" t="s">
-        <v>106</v>
-      </c>
-      <c r="B81" t="s">
-        <v>163</v>
-      </c>
-      <c r="C81" t="s">
-        <v>12</v>
-      </c>
-      <c r="D81">
-        <v>9</v>
-      </c>
       <c r="E81" t="s">
-        <v>8</v>
+        <v>97</v>
       </c>
       <c r="F81" t="s">
-        <v>152</v>
-      </c>
-      <c r="G81">
-        <v>57600000</v>
+        <v>15</v>
+      </c>
+      <c r="G81" s="6">
+        <v>21300000</v>
       </c>
       <c r="I81">
-        <v>7200</v>
+        <v>4125</v>
       </c>
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>108</v>
+        <v>147</v>
       </c>
       <c r="B82" t="s">
-        <v>164</v>
+        <v>148</v>
       </c>
       <c r="C82" t="s">
         <v>7</v>
       </c>
       <c r="D82">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="E82" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="F82" t="s">
-        <v>152</v>
+        <v>15</v>
       </c>
       <c r="G82">
-        <v>48000000</v>
+        <v>20800000</v>
       </c>
       <c r="I82">
-        <v>9600</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>146</v>
+        <v>105</v>
       </c>
       <c r="B83" t="s">
-        <v>165</v>
+        <v>149</v>
       </c>
       <c r="C83" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="D83">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E83" t="s">
-        <v>98</v>
+        <v>8</v>
       </c>
       <c r="F83" t="s">
-        <v>152</v>
+        <v>15</v>
       </c>
       <c r="G83">
-        <v>16800000</v>
+        <v>64800000</v>
       </c>
       <c r="I83">
-        <v>3200</v>
+        <v>7200</v>
       </c>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
+        <v>143</v>
+      </c>
+      <c r="B84" t="s">
         <v>150</v>
       </c>
-      <c r="B84" t="s">
-        <v>166</v>
-      </c>
       <c r="C84" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="D84">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="E84" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F84" t="s">
-        <v>152</v>
+        <v>15</v>
       </c>
       <c r="G84">
-        <v>37440000</v>
+        <v>10560000</v>
       </c>
       <c r="I84">
-        <v>7200</v>
+        <v>3200</v>
       </c>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>150</v>
+        <v>109</v>
       </c>
       <c r="B85" t="s">
-        <v>167</v>
+        <v>151</v>
       </c>
       <c r="C85" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="D85">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="E85" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="F85" t="s">
-        <v>155</v>
+        <v>15</v>
       </c>
       <c r="G85">
-        <v>21600000</v>
+        <v>3520000</v>
       </c>
       <c r="I85">
-        <v>7200</v>
+        <v>800</v>
       </c>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="B86" t="s">
-        <v>168</v>
+        <v>152</v>
       </c>
       <c r="C86" t="s">
         <v>7</v>
       </c>
       <c r="D86">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E86" t="s">
-        <v>8</v>
+        <v>97</v>
       </c>
       <c r="F86" t="s">
-        <v>152</v>
+        <v>181</v>
       </c>
       <c r="G86">
-        <v>36000000</v>
+        <v>7560000</v>
       </c>
       <c r="I86">
-        <v>4000</v>
+        <v>2400</v>
       </c>
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="B87" t="s">
-        <v>169</v>
+        <v>153</v>
       </c>
       <c r="C87" t="s">
         <v>7</v>
       </c>
       <c r="D87">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E87" t="s">
         <v>8</v>
       </c>
       <c r="F87" t="s">
-        <v>152</v>
+        <v>15</v>
       </c>
       <c r="G87">
-        <v>72000000</v>
+        <v>91200000</v>
       </c>
       <c r="I87">
-        <v>8000</v>
+        <v>9600</v>
       </c>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>105</v>
+        <v>154</v>
       </c>
       <c r="B88" t="s">
-        <v>170</v>
+        <v>155</v>
       </c>
       <c r="C88" t="s">
-        <v>7</v>
+        <v>58</v>
       </c>
       <c r="D88">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E88" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="F88" t="s">
-        <v>152</v>
+        <v>15</v>
       </c>
       <c r="G88">
-        <v>12480000</v>
+        <v>28800000</v>
       </c>
       <c r="I88">
-        <v>2400</v>
+        <v>4800</v>
       </c>
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>105</v>
+        <v>154</v>
       </c>
       <c r="B89" t="s">
-        <v>171</v>
+        <v>156</v>
       </c>
       <c r="C89" t="s">
-        <v>7</v>
+        <v>58</v>
       </c>
       <c r="D89">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E89" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="F89" t="s">
-        <v>152</v>
+        <v>15</v>
       </c>
       <c r="G89">
-        <v>16640000</v>
+        <v>9600000</v>
       </c>
       <c r="I89">
-        <v>3200</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B90" t="s">
-        <v>172</v>
+        <v>157</v>
       </c>
       <c r="C90" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="D90">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="E90" t="s">
-        <v>8</v>
+        <v>96</v>
       </c>
       <c r="F90" t="s">
-        <v>152</v>
+        <v>15</v>
       </c>
       <c r="G90">
-        <v>80640000</v>
+        <v>20800000</v>
       </c>
       <c r="I90">
-        <v>9600</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>159</v>
+        <v>103</v>
       </c>
       <c r="B91" t="s">
-        <v>173</v>
+        <v>158</v>
       </c>
       <c r="C91" t="s">
-        <v>59</v>
+        <v>12</v>
       </c>
       <c r="D91">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E91" t="s">
-        <v>99</v>
+        <v>8</v>
       </c>
       <c r="F91" t="s">
-        <v>155</v>
+        <v>15</v>
       </c>
       <c r="G91">
-        <v>17280000</v>
+        <v>57600000</v>
       </c>
       <c r="I91">
-        <v>4800</v>
+        <v>7200</v>
       </c>
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B92" t="s">
-        <v>174</v>
+        <v>159</v>
       </c>
       <c r="C92" t="s">
         <v>7</v>
       </c>
       <c r="D92">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="E92" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="F92" t="s">
-        <v>152</v>
+        <v>15</v>
       </c>
       <c r="G92">
-        <v>20800000</v>
+        <v>48000000</v>
       </c>
       <c r="I92">
-        <v>4000</v>
+        <v>9600</v>
       </c>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>107</v>
+        <v>143</v>
       </c>
       <c r="B93" t="s">
-        <v>175</v>
+        <v>160</v>
       </c>
       <c r="C93" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="D93">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E93" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="F93" t="s">
-        <v>155</v>
+        <v>15</v>
       </c>
       <c r="G93">
-        <v>12000000</v>
+        <v>16800000</v>
       </c>
       <c r="I93">
-        <v>4000</v>
+        <v>3200</v>
       </c>
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>104</v>
+        <v>147</v>
       </c>
       <c r="B94" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="C94" t="s">
         <v>7</v>
       </c>
       <c r="D94">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E94" t="s">
-        <v>8</v>
+        <v>96</v>
       </c>
       <c r="F94" t="s">
-        <v>152</v>
+        <v>15</v>
       </c>
       <c r="G94">
-        <v>91200000</v>
+        <v>37440000</v>
       </c>
       <c r="I94">
-        <v>9600</v>
+        <v>7200</v>
       </c>
     </row>
     <row r="95" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>104</v>
+        <v>147</v>
       </c>
       <c r="B95" t="s">
-        <v>177</v>
+        <v>162</v>
       </c>
       <c r="C95" t="s">
         <v>7</v>
@@ -3581,13 +3670,13 @@
         <v>9</v>
       </c>
       <c r="E95" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F95" t="s">
-        <v>152</v>
+        <v>181</v>
       </c>
       <c r="G95">
-        <v>37440000</v>
+        <v>21600000</v>
       </c>
       <c r="I95">
         <v>7200</v>
@@ -3595,28 +3684,28 @@
     </row>
     <row r="96" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B96" t="s">
-        <v>178</v>
+        <v>163</v>
       </c>
       <c r="C96" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="D96">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E96" t="s">
-        <v>98</v>
+        <v>8</v>
       </c>
       <c r="F96" t="s">
-        <v>152</v>
+        <v>15</v>
       </c>
       <c r="G96">
-        <v>16800000</v>
+        <v>36000000</v>
       </c>
       <c r="I96">
-        <v>3200</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.25">
@@ -3624,179 +3713,449 @@
         <v>105</v>
       </c>
       <c r="B97" t="s">
-        <v>179</v>
+        <v>164</v>
       </c>
       <c r="C97" t="s">
         <v>7</v>
       </c>
       <c r="D97">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E97" t="s">
         <v>8</v>
       </c>
       <c r="F97" t="s">
-        <v>152</v>
+        <v>15</v>
       </c>
       <c r="G97">
-        <v>36000000</v>
+        <v>72000000</v>
       </c>
       <c r="I97">
-        <v>4000</v>
+        <v>8000</v>
       </c>
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B98" t="s">
-        <v>180</v>
+        <v>165</v>
       </c>
       <c r="C98" t="s">
         <v>7</v>
       </c>
       <c r="D98">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E98" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="F98" t="s">
-        <v>152</v>
+        <v>15</v>
       </c>
       <c r="G98">
-        <v>41600000</v>
+        <v>12480000</v>
       </c>
       <c r="I98">
-        <v>8000</v>
+        <v>2400</v>
       </c>
     </row>
     <row r="99" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B99" t="s">
-        <v>181</v>
+        <v>166</v>
       </c>
       <c r="C99" t="s">
         <v>7</v>
       </c>
       <c r="D99">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E99" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="F99" t="s">
-        <v>155</v>
+        <v>15</v>
       </c>
       <c r="G99">
-        <v>7200000</v>
+        <v>16640000</v>
       </c>
       <c r="I99">
-        <v>2400</v>
+        <v>3200</v>
       </c>
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B100" t="s">
-        <v>182</v>
+        <v>167</v>
       </c>
       <c r="C100" t="s">
         <v>12</v>
       </c>
       <c r="D100">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E100" t="s">
-        <v>98</v>
+        <v>8</v>
       </c>
       <c r="F100" t="s">
-        <v>152</v>
+        <v>15</v>
       </c>
       <c r="G100">
-        <v>37440000</v>
+        <v>80640000</v>
       </c>
       <c r="I100">
-        <v>7200</v>
+        <v>9600</v>
       </c>
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>108</v>
+        <v>154</v>
       </c>
       <c r="B101" t="s">
-        <v>183</v>
+        <v>168</v>
       </c>
       <c r="C101" t="s">
+        <v>58</v>
+      </c>
+      <c r="D101">
+        <v>6</v>
+      </c>
+      <c r="E101" t="s">
+        <v>97</v>
+      </c>
+      <c r="F101" t="s">
+        <v>181</v>
+      </c>
+      <c r="G101">
+        <v>17280000</v>
+      </c>
+      <c r="I101">
+        <v>4800</v>
+      </c>
+    </row>
+    <row r="102" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>104</v>
+      </c>
+      <c r="B102" t="s">
+        <v>169</v>
+      </c>
+      <c r="C102" t="s">
+        <v>7</v>
+      </c>
+      <c r="D102">
+        <v>5</v>
+      </c>
+      <c r="E102" t="s">
+        <v>96</v>
+      </c>
+      <c r="F102" t="s">
+        <v>15</v>
+      </c>
+      <c r="G102">
+        <v>20800000</v>
+      </c>
+      <c r="I102">
+        <v>4000</v>
+      </c>
+    </row>
+    <row r="103" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>104</v>
+      </c>
+      <c r="B103" t="s">
+        <v>170</v>
+      </c>
+      <c r="C103" t="s">
+        <v>7</v>
+      </c>
+      <c r="D103">
+        <v>5</v>
+      </c>
+      <c r="E103" t="s">
+        <v>97</v>
+      </c>
+      <c r="F103" t="s">
+        <v>181</v>
+      </c>
+      <c r="G103">
+        <v>12000000</v>
+      </c>
+      <c r="I103">
+        <v>4000</v>
+      </c>
+    </row>
+    <row r="104" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>101</v>
+      </c>
+      <c r="B104" t="s">
+        <v>171</v>
+      </c>
+      <c r="C104" t="s">
+        <v>7</v>
+      </c>
+      <c r="D104">
+        <v>12</v>
+      </c>
+      <c r="E104" t="s">
+        <v>8</v>
+      </c>
+      <c r="F104" t="s">
+        <v>15</v>
+      </c>
+      <c r="G104">
+        <v>91200000</v>
+      </c>
+      <c r="I104">
+        <v>9600</v>
+      </c>
+    </row>
+    <row r="105" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>101</v>
+      </c>
+      <c r="B105" t="s">
+        <v>172</v>
+      </c>
+      <c r="C105" t="s">
+        <v>7</v>
+      </c>
+      <c r="D105">
+        <v>9</v>
+      </c>
+      <c r="E105" t="s">
+        <v>96</v>
+      </c>
+      <c r="F105" t="s">
+        <v>15</v>
+      </c>
+      <c r="G105">
+        <v>37440000</v>
+      </c>
+      <c r="I105">
+        <v>7200</v>
+      </c>
+    </row>
+    <row r="106" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>101</v>
+      </c>
+      <c r="B106" t="s">
+        <v>173</v>
+      </c>
+      <c r="C106" t="s">
+        <v>14</v>
+      </c>
+      <c r="D106">
+        <v>4</v>
+      </c>
+      <c r="E106" t="s">
+        <v>96</v>
+      </c>
+      <c r="F106" t="s">
+        <v>15</v>
+      </c>
+      <c r="G106">
+        <v>16800000</v>
+      </c>
+      <c r="I106">
+        <v>3200</v>
+      </c>
+    </row>
+    <row r="107" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>102</v>
+      </c>
+      <c r="B107" t="s">
+        <v>174</v>
+      </c>
+      <c r="C107" t="s">
+        <v>7</v>
+      </c>
+      <c r="D107">
+        <v>5</v>
+      </c>
+      <c r="E107" t="s">
+        <v>8</v>
+      </c>
+      <c r="F107" t="s">
+        <v>15</v>
+      </c>
+      <c r="G107">
+        <v>36000000</v>
+      </c>
+      <c r="I107">
+        <v>4000</v>
+      </c>
+    </row>
+    <row r="108" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>102</v>
+      </c>
+      <c r="B108" t="s">
+        <v>175</v>
+      </c>
+      <c r="C108" t="s">
+        <v>7</v>
+      </c>
+      <c r="D108">
+        <v>10</v>
+      </c>
+      <c r="E108" t="s">
+        <v>96</v>
+      </c>
+      <c r="F108" t="s">
+        <v>15</v>
+      </c>
+      <c r="G108">
+        <v>41600000</v>
+      </c>
+      <c r="I108">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="109" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>102</v>
+      </c>
+      <c r="B109" t="s">
+        <v>176</v>
+      </c>
+      <c r="C109" t="s">
+        <v>7</v>
+      </c>
+      <c r="D109">
+        <v>3</v>
+      </c>
+      <c r="E109" t="s">
+        <v>97</v>
+      </c>
+      <c r="F109" t="s">
+        <v>181</v>
+      </c>
+      <c r="G109">
+        <v>7200000</v>
+      </c>
+      <c r="I109">
+        <v>2400</v>
+      </c>
+    </row>
+    <row r="110" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>102</v>
+      </c>
+      <c r="B110" t="s">
+        <v>177</v>
+      </c>
+      <c r="C110" t="s">
+        <v>12</v>
+      </c>
+      <c r="D110">
+        <v>9</v>
+      </c>
+      <c r="E110" t="s">
+        <v>96</v>
+      </c>
+      <c r="F110" t="s">
+        <v>15</v>
+      </c>
+      <c r="G110">
+        <v>37440000</v>
+      </c>
+      <c r="I110">
+        <v>7200</v>
+      </c>
+    </row>
+    <row r="111" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>105</v>
+      </c>
+      <c r="B111" t="s">
+        <v>178</v>
+      </c>
+      <c r="C111" t="s">
         <v>17</v>
       </c>
-      <c r="D101">
+      <c r="D111">
         <v>9</v>
       </c>
-      <c r="E101" t="s">
-        <v>8</v>
-      </c>
-      <c r="F101" t="s">
-        <v>152</v>
-      </c>
-      <c r="G101">
+      <c r="E111" t="s">
+        <v>8</v>
+      </c>
+      <c r="F111" t="s">
+        <v>15</v>
+      </c>
+      <c r="G111">
         <v>60480000</v>
       </c>
-      <c r="I101">
+      <c r="I111">
         <v>7200</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B2:H41">
-    <sortCondition ref="B1:B41"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:I51">
+    <sortCondition ref="A2:A51"/>
   </sortState>
   <hyperlinks>
-    <hyperlink ref="H34" r:id="rId1" display="https://prozorro.gov.ua/tender/UA-2023-10-11-014375-a" xr:uid="{CC830BD6-390C-465E-94E5-E5E7341F3B7F}"/>
+    <hyperlink ref="H44" r:id="rId1" display="https://prozorro.gov.ua/tender/UA-2023-10-11-014375-a" xr:uid="{CC830BD6-390C-465E-94E5-E5E7341F3B7F}"/>
     <hyperlink ref="H7" r:id="rId2" xr:uid="{E6277324-1B9E-41B9-986E-B780472883E5}"/>
     <hyperlink ref="H8" r:id="rId3" xr:uid="{890EB980-9C16-4888-881E-D7568A3050BD}"/>
     <hyperlink ref="H11" r:id="rId4" xr:uid="{76E5BABA-C6CC-480D-A8BC-3C424BD409C2}"/>
     <hyperlink ref="H4" r:id="rId5" xr:uid="{8B9FF1EF-73A8-439D-90B6-3DCA3D6A75CC}"/>
     <hyperlink ref="H10" r:id="rId6" xr:uid="{1512864A-61CE-41C1-92FF-2FDCFD04AF97}"/>
-    <hyperlink ref="H36" r:id="rId7" xr:uid="{4B99C35A-02C3-4BC9-8EE0-990E49A5FCBD}"/>
-    <hyperlink ref="H14" r:id="rId8" xr:uid="{821DFB83-ED7B-4B63-9555-14A846AFE00D}"/>
+    <hyperlink ref="H46" r:id="rId7" xr:uid="{4B99C35A-02C3-4BC9-8EE0-990E49A5FCBD}"/>
+    <hyperlink ref="H17" r:id="rId8" xr:uid="{821DFB83-ED7B-4B63-9555-14A846AFE00D}"/>
     <hyperlink ref="H9" r:id="rId9" xr:uid="{BA78665F-5EB1-4DEF-9D7D-9841133DA028}"/>
     <hyperlink ref="H5" r:id="rId10" display="https://prozorro.gov.ua/tender/UA-2023-07-27-009934-a" xr:uid="{94AC0BB1-8607-436A-A8F2-548E7E654B0E}"/>
     <hyperlink ref="H3" r:id="rId11" display="https://prozorro.gov.ua/tender/UA-2023-07-27-009550-a" xr:uid="{C7E1EB43-7FB9-4CF9-9C84-7F5AA608DF3F}"/>
-    <hyperlink ref="H13" r:id="rId12" xr:uid="{A3FCEB43-9C7B-4ACB-8DE5-00AD1A9A6D52}"/>
-    <hyperlink ref="H12" r:id="rId13" xr:uid="{AC0D3914-0FB8-4DD8-9FCF-AE17A48744C6}"/>
-    <hyperlink ref="H32" r:id="rId14" xr:uid="{2E7C2A7E-6D85-438E-A957-4E8B4A48BAF6}"/>
-    <hyperlink ref="H38" r:id="rId15" xr:uid="{0CE4654C-C13D-45A6-9904-1460BBF1D7FA}"/>
-    <hyperlink ref="H22" r:id="rId16" xr:uid="{E0E9B52B-F080-4081-9F8D-59409CC02214}"/>
-    <hyperlink ref="H23" r:id="rId17" xr:uid="{8ADB3CD8-B9D5-4852-BC40-F0AF25EEB092}"/>
-    <hyperlink ref="H24" r:id="rId18" xr:uid="{D368785C-5CFA-4C46-900A-7C5A3814640B}"/>
-    <hyperlink ref="H25" r:id="rId19" xr:uid="{578BF64D-EBBE-4FE0-98A3-6CD16BB6149D}"/>
-    <hyperlink ref="H26" r:id="rId20" xr:uid="{849AEA57-84A7-4DCF-99C0-489A2B345F18}"/>
-    <hyperlink ref="H27" r:id="rId21" xr:uid="{D2A19AB9-1C37-4007-84F4-F3B9EADBE701}"/>
-    <hyperlink ref="H35" r:id="rId22" xr:uid="{8D7D301C-66D7-411C-BAF0-CC8A335F69C5}"/>
-    <hyperlink ref="H37" r:id="rId23" xr:uid="{DFC1E3BD-6ED8-433C-8407-7833FDBB5AA7}"/>
-    <hyperlink ref="H28" r:id="rId24" xr:uid="{D893FF3C-BA47-4123-84CE-C0565D1D1816}"/>
-    <hyperlink ref="H31" r:id="rId25" xr:uid="{E1FAC06D-FF2F-4A68-800E-6A0F38CB4ED5}"/>
-    <hyperlink ref="H33" r:id="rId26" xr:uid="{27A90131-F6AF-4714-85C1-5DD820F41084}"/>
-    <hyperlink ref="H18" r:id="rId27" xr:uid="{FFF1E74C-83E0-40F1-AF8E-8BB317400EA3}"/>
-    <hyperlink ref="H21" r:id="rId28" xr:uid="{1B321A70-2863-44C8-9F1F-8AC5BAD04FDE}"/>
-    <hyperlink ref="H19" r:id="rId29" xr:uid="{FAEC6FA8-5D02-4EF8-B7BC-4769CD1D66E9}"/>
-    <hyperlink ref="H20" r:id="rId30" xr:uid="{1F48BA6C-7386-42D9-A319-35A52B5F0E21}"/>
-    <hyperlink ref="H30" r:id="rId31" xr:uid="{8F6C5CD4-96D2-45FE-9DB2-67D301A9AA04}"/>
-    <hyperlink ref="H29" r:id="rId32" xr:uid="{E5140C6D-CF55-40E9-B930-DCF595012511}"/>
+    <hyperlink ref="H16" r:id="rId12" xr:uid="{A3FCEB43-9C7B-4ACB-8DE5-00AD1A9A6D52}"/>
+    <hyperlink ref="H15" r:id="rId13" xr:uid="{AC0D3914-0FB8-4DD8-9FCF-AE17A48744C6}"/>
+    <hyperlink ref="H42" r:id="rId14" xr:uid="{2E7C2A7E-6D85-438E-A957-4E8B4A48BAF6}"/>
+    <hyperlink ref="H49" r:id="rId15" xr:uid="{0CE4654C-C13D-45A6-9904-1460BBF1D7FA}"/>
+    <hyperlink ref="H32" r:id="rId16" xr:uid="{E0E9B52B-F080-4081-9F8D-59409CC02214}"/>
+    <hyperlink ref="H33" r:id="rId17" xr:uid="{8ADB3CD8-B9D5-4852-BC40-F0AF25EEB092}"/>
+    <hyperlink ref="H34" r:id="rId18" xr:uid="{D368785C-5CFA-4C46-900A-7C5A3814640B}"/>
+    <hyperlink ref="H35" r:id="rId19" xr:uid="{578BF64D-EBBE-4FE0-98A3-6CD16BB6149D}"/>
+    <hyperlink ref="H36" r:id="rId20" xr:uid="{849AEA57-84A7-4DCF-99C0-489A2B345F18}"/>
+    <hyperlink ref="H37" r:id="rId21" xr:uid="{D2A19AB9-1C37-4007-84F4-F3B9EADBE701}"/>
+    <hyperlink ref="H45" r:id="rId22" xr:uid="{8D7D301C-66D7-411C-BAF0-CC8A335F69C5}"/>
+    <hyperlink ref="H47" r:id="rId23" xr:uid="{DFC1E3BD-6ED8-433C-8407-7833FDBB5AA7}"/>
+    <hyperlink ref="H38" r:id="rId24" xr:uid="{D893FF3C-BA47-4123-84CE-C0565D1D1816}"/>
+    <hyperlink ref="H41" r:id="rId25" xr:uid="{E1FAC06D-FF2F-4A68-800E-6A0F38CB4ED5}"/>
+    <hyperlink ref="H43" r:id="rId26" xr:uid="{27A90131-F6AF-4714-85C1-5DD820F41084}"/>
+    <hyperlink ref="H28" r:id="rId27" xr:uid="{FFF1E74C-83E0-40F1-AF8E-8BB317400EA3}"/>
+    <hyperlink ref="H31" r:id="rId28" xr:uid="{1B321A70-2863-44C8-9F1F-8AC5BAD04FDE}"/>
+    <hyperlink ref="H29" r:id="rId29" xr:uid="{FAEC6FA8-5D02-4EF8-B7BC-4769CD1D66E9}"/>
+    <hyperlink ref="H30" r:id="rId30" xr:uid="{1F48BA6C-7386-42D9-A319-35A52B5F0E21}"/>
+    <hyperlink ref="H40" r:id="rId31" xr:uid="{8F6C5CD4-96D2-45FE-9DB2-67D301A9AA04}"/>
+    <hyperlink ref="H39" r:id="rId32" xr:uid="{E5140C6D-CF55-40E9-B930-DCF595012511}"/>
     <hyperlink ref="H6" r:id="rId33" xr:uid="{5CDA56AC-FABF-471E-88E1-1A526DBEACA8}"/>
-    <hyperlink ref="H15" r:id="rId34" xr:uid="{CE0FD1F9-8126-4F9B-92BB-816DAA21203D}"/>
-    <hyperlink ref="H16" r:id="rId35" xr:uid="{15DF762F-41C8-45AF-BEED-1F9D5F50D852}"/>
-    <hyperlink ref="H39" r:id="rId36" xr:uid="{193EDECE-04EE-4DA0-9F3C-CE8F5766608B}"/>
-    <hyperlink ref="H40" r:id="rId37" xr:uid="{D7966B98-AD1E-4714-BEE3-CE3CF6EC2D08}"/>
-    <hyperlink ref="H41" r:id="rId38" xr:uid="{795E7A1B-94F3-481B-A0D2-B90199638357}"/>
-    <hyperlink ref="H2" r:id="rId39" xr:uid="{7090DC7F-89B1-42E7-B933-A4C725EFE1ED}"/>
-    <hyperlink ref="H17" r:id="rId40" xr:uid="{9BDC4451-1FBA-4CB5-9E51-2CE6FE340C83}"/>
+    <hyperlink ref="H18" r:id="rId34" xr:uid="{CE0FD1F9-8126-4F9B-92BB-816DAA21203D}"/>
+    <hyperlink ref="H50" r:id="rId35" xr:uid="{193EDECE-04EE-4DA0-9F3C-CE8F5766608B}"/>
+    <hyperlink ref="H51" r:id="rId36" xr:uid="{D7966B98-AD1E-4714-BEE3-CE3CF6EC2D08}"/>
+    <hyperlink ref="H2" r:id="rId37" xr:uid="{7090DC7F-89B1-42E7-B933-A4C725EFE1ED}"/>
+    <hyperlink ref="H27" r:id="rId38" xr:uid="{9BDC4451-1FBA-4CB5-9E51-2CE6FE340C83}"/>
+    <hyperlink ref="H19" r:id="rId39" xr:uid="{4A29D3B0-3C65-4EAC-BA5C-5B9CAC14683C}"/>
+    <hyperlink ref="H20" r:id="rId40" xr:uid="{7EE78492-9322-4FAE-9434-B9BD8A8D6CE7}"/>
+    <hyperlink ref="H21" r:id="rId41" xr:uid="{1182108E-C42B-4C30-BAE7-B4AEED1B7E87}"/>
+    <hyperlink ref="H22" r:id="rId42" xr:uid="{BF78DCE1-F559-4A00-87A0-3DB441896577}"/>
+    <hyperlink ref="H23" r:id="rId43" xr:uid="{1CF082EC-19D0-4B90-9FB0-42D934A8571C}"/>
+    <hyperlink ref="H24" r:id="rId44" xr:uid="{71E41883-655E-4EAA-AB5D-BC157BF1E443}"/>
+    <hyperlink ref="H25" r:id="rId45" xr:uid="{CBFB43FD-A3B9-4188-A49D-F300E14C6FAF}"/>
+    <hyperlink ref="H26" r:id="rId46" xr:uid="{9FC58DFE-D6D2-47DB-9F28-8826DBDEA9D8}"/>
+    <hyperlink ref="H13" r:id="rId47" xr:uid="{F84AEAA7-EC22-4D5C-BF9F-1CED353C41C0}"/>
+    <hyperlink ref="H14" r:id="rId48" xr:uid="{5F5E15DD-B1E2-4CB0-B242-37C28A8B7E12}"/>
+    <hyperlink ref="H12" r:id="rId49" xr:uid="{98031769-532F-47C6-8210-C4D540B2462D}"/>
+    <hyperlink ref="H48" r:id="rId50" xr:uid="{CF20909E-DC64-43BD-B284-9C2194E4D872}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId41"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId51"/>
 </worksheet>
 </file>
 
@@ -3817,7 +4176,7 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: trained model again with new repair types
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\personal\Аспирантура\Статьи\Стаття інформ. сист\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projects\python\corruption-risks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88FCAF65-7510-4B02-891A-9E8175A87192}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB2F3848-0514-4469-9F9F-3D2F152436C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -318,9 +318,6 @@
     <t>UA-2023-07-28-005566-a</t>
   </si>
   <si>
-    <t> м. Одеса, вул. Середня, 24</t>
-  </si>
-  <si>
     <t>UA-2024-08-30-007696-a</t>
   </si>
   <si>
@@ -649,6 +646,9 @@
   </si>
   <si>
     <t>м. Харків, пр. Аерокосмічний, 21</t>
+  </si>
+  <si>
+    <t> м. Одеса, вул.Косовська, 2-Д</t>
   </si>
 </sst>
 </file>
@@ -725,7 +725,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -750,15 +750,10 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Гиперссылка" xfId="1" builtinId="8"/>
-    <cellStyle name="Обычный" xfId="0" builtinId="0"/>
+    <cellStyle name="Гіперпосилання" xfId="1" builtinId="8"/>
+    <cellStyle name="Звичайний" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1051,7 +1046,7 @@
   <sheetData>
     <row r="1" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>0</v>
@@ -1075,15 +1070,15 @@
         <v>6</v>
       </c>
       <c r="I1" s="9" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B2" t="s">
-        <v>92</v>
+        <v>202</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>7</v>
@@ -1101,7 +1096,7 @@
         <v>32788802</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="I2">
         <v>4000</v>
@@ -1109,7 +1104,7 @@
     </row>
     <row r="3" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>29</v>
@@ -1138,7 +1133,7 @@
     </row>
     <row r="4" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>28</v>
@@ -1150,7 +1145,7 @@
         <v>9</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>15</v>
@@ -1167,7 +1162,7 @@
     </row>
     <row r="5" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>26</v>
@@ -1196,7 +1191,7 @@
     </row>
     <row r="6" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>72</v>
@@ -1225,7 +1220,7 @@
     </row>
     <row r="7" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>24</v>
@@ -1254,7 +1249,7 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>74</v>
@@ -1283,7 +1278,7 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>80</v>
@@ -1312,7 +1307,7 @@
     </row>
     <row r="10" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>77</v>
@@ -1341,10 +1336,10 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>7</v>
@@ -1369,95 +1364,95 @@
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12" s="10" t="s">
-        <v>102</v>
-      </c>
-      <c r="B12" s="10" t="s">
+      <c r="A12" t="s">
+        <v>101</v>
+      </c>
+      <c r="B12" t="s">
+        <v>197</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12" s="1">
+        <v>9</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="F12" t="s">
+        <v>15</v>
+      </c>
+      <c r="G12" s="6">
+        <v>57624052</v>
+      </c>
+      <c r="H12" s="4" t="s">
         <v>198</v>
       </c>
-      <c r="C12" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="D12" s="11">
+      <c r="I12">
+        <v>7200</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>146</v>
+      </c>
+      <c r="B13" t="s">
+        <v>193</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D13" s="1">
         <v>9</v>
       </c>
-      <c r="E12" s="11" t="s">
-        <v>96</v>
-      </c>
-      <c r="F12" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="G12" s="12">
-        <v>57624052</v>
-      </c>
-      <c r="H12" s="4" t="s">
-        <v>199</v>
-      </c>
-      <c r="I12" s="10">
+      <c r="E13" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F13" t="s">
+        <v>15</v>
+      </c>
+      <c r="G13" s="6">
+        <v>84999841</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="I13">
         <v>7200</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" s="10" t="s">
-        <v>147</v>
-      </c>
-      <c r="B13" s="10" t="s">
-        <v>194</v>
-      </c>
-      <c r="C13" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="D13" s="11">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>146</v>
+      </c>
+      <c r="B14" t="s">
+        <v>195</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D14" s="1">
         <v>9</v>
       </c>
-      <c r="E13" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="F13" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="G13" s="12">
-        <v>84999841</v>
-      </c>
-      <c r="H13" s="4" t="s">
-        <v>195</v>
-      </c>
-      <c r="I13" s="10">
-        <v>7200</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A14" s="10" t="s">
-        <v>147</v>
-      </c>
-      <c r="B14" s="10" t="s">
+      <c r="E14" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="F14" t="s">
+        <v>15</v>
+      </c>
+      <c r="G14" s="6">
+        <v>36595864</v>
+      </c>
+      <c r="H14" s="4" t="s">
         <v>196</v>
       </c>
-      <c r="C14" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="D14" s="11">
-        <v>9</v>
-      </c>
-      <c r="E14" s="11" t="s">
-        <v>96</v>
-      </c>
-      <c r="F14" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="G14" s="12">
-        <v>36595864</v>
-      </c>
-      <c r="H14" s="4" t="s">
-        <v>197</v>
-      </c>
-      <c r="I14" s="10">
+      <c r="I14">
         <v>7200</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>21</v>
@@ -1486,7 +1481,7 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>20</v>
@@ -1498,7 +1493,7 @@
         <v>9</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F16" s="1" t="s">
         <v>15</v>
@@ -1515,7 +1510,7 @@
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>16</v>
@@ -1527,7 +1522,7 @@
         <v>5</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F17" s="1" t="s">
         <v>15</v>
@@ -1544,7 +1539,7 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>84</v>
@@ -1556,7 +1551,7 @@
         <v>5</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F18" s="1" t="s">
         <v>15</v>
@@ -1572,240 +1567,240 @@
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19" s="10" t="s">
-        <v>103</v>
-      </c>
-      <c r="B19" s="10" t="s">
+      <c r="A19" t="s">
+        <v>102</v>
+      </c>
+      <c r="B19" t="s">
+        <v>178</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D19" s="1">
+        <v>9</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F19" t="s">
+        <v>15</v>
+      </c>
+      <c r="G19" s="6">
+        <v>91668437</v>
+      </c>
+      <c r="H19" s="4" t="s">
         <v>179</v>
       </c>
-      <c r="C19" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="D19" s="11">
-        <v>9</v>
-      </c>
-      <c r="E19" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="F19" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="G19" s="12">
-        <v>91668437</v>
-      </c>
-      <c r="H19" s="4" t="s">
-        <v>180</v>
-      </c>
-      <c r="I19" s="10">
+      <c r="I19">
         <v>7200</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="10" t="s">
-        <v>103</v>
-      </c>
-      <c r="B20" s="10" t="s">
+      <c r="A20" t="s">
+        <v>102</v>
+      </c>
+      <c r="B20" t="s">
+        <v>181</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20" s="1">
+        <v>5</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" t="s">
+        <v>15</v>
+      </c>
+      <c r="G20" s="6">
+        <v>56753765</v>
+      </c>
+      <c r="H20" s="4" t="s">
         <v>182</v>
       </c>
-      <c r="C20" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="D20" s="11">
+      <c r="I20">
+        <v>4000</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>102</v>
+      </c>
+      <c r="B21" t="s">
+        <v>183</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D21" s="1">
+        <v>3</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F21" t="s">
+        <v>15</v>
+      </c>
+      <c r="G21" s="6">
+        <v>50488018</v>
+      </c>
+      <c r="H21" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="I21">
+        <v>2400</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>102</v>
+      </c>
+      <c r="B22" t="s">
+        <v>185</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D22" s="1">
+        <v>4</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F22" t="s">
+        <v>15</v>
+      </c>
+      <c r="G22" s="6">
+        <v>64471674</v>
+      </c>
+      <c r="H22" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="I22">
+        <v>3200</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>102</v>
+      </c>
+      <c r="B23" t="s">
+        <v>94</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D23" s="1">
         <v>5</v>
       </c>
-      <c r="E20" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="F20" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="G20" s="12">
-        <v>56753765</v>
-      </c>
-      <c r="H20" s="4" t="s">
-        <v>183</v>
-      </c>
-      <c r="I20" s="10">
-        <v>4000</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A21" s="10" t="s">
-        <v>103</v>
-      </c>
-      <c r="B21" s="10" t="s">
-        <v>184</v>
-      </c>
-      <c r="C21" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="D21" s="11">
-        <v>3</v>
-      </c>
-      <c r="E21" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="F21" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="G21" s="12">
-        <v>50488018</v>
-      </c>
-      <c r="H21" s="4" t="s">
-        <v>185</v>
-      </c>
-      <c r="I21" s="10">
-        <v>2400</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A22" s="10" t="s">
-        <v>103</v>
-      </c>
-      <c r="B22" s="10" t="s">
-        <v>186</v>
-      </c>
-      <c r="C22" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="D22" s="11">
-        <v>4</v>
-      </c>
-      <c r="E22" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="F22" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="G22" s="12">
-        <v>64471674</v>
-      </c>
-      <c r="H22" s="4" t="s">
-        <v>187</v>
-      </c>
-      <c r="I22" s="10">
-        <v>3200</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A23" s="10" t="s">
-        <v>103</v>
-      </c>
-      <c r="B23" s="10" t="s">
-        <v>95</v>
-      </c>
-      <c r="C23" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="D23" s="11">
-        <v>5</v>
-      </c>
-      <c r="E23" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="F23" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="G23" s="12">
+      <c r="E23" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F23" t="s">
+        <v>15</v>
+      </c>
+      <c r="G23" s="6">
         <v>139636363</v>
       </c>
       <c r="H23" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="I23" s="10">
+      <c r="I23">
         <v>4000</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A24" s="10" t="s">
-        <v>103</v>
-      </c>
-      <c r="B24" s="10" t="s">
+      <c r="A24" t="s">
+        <v>102</v>
+      </c>
+      <c r="B24" t="s">
+        <v>187</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D24" s="1">
+        <v>5</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F24" t="s">
+        <v>15</v>
+      </c>
+      <c r="G24" s="6">
+        <v>214180976</v>
+      </c>
+      <c r="H24" s="4" t="s">
         <v>188</v>
       </c>
-      <c r="C24" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="D24" s="11">
+      <c r="I24">
+        <v>4000</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>102</v>
+      </c>
+      <c r="B25" t="s">
+        <v>190</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D25" s="1">
         <v>5</v>
       </c>
-      <c r="E24" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="F24" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="G24" s="12">
-        <v>214180976</v>
-      </c>
-      <c r="H24" s="4" t="s">
+      <c r="E25" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F25" t="s">
+        <v>15</v>
+      </c>
+      <c r="G25" s="6">
+        <v>162165984</v>
+      </c>
+      <c r="H25" s="4" t="s">
         <v>189</v>
       </c>
-      <c r="I24" s="10">
+      <c r="I25">
         <v>4000</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" s="10" t="s">
-        <v>103</v>
-      </c>
-      <c r="B25" s="10" t="s">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>102</v>
+      </c>
+      <c r="B26" t="s">
         <v>191</v>
       </c>
-      <c r="C25" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="D25" s="11">
+      <c r="C26" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D26" s="1">
         <v>5</v>
       </c>
-      <c r="E25" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="F25" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="G25" s="12">
-        <v>162165984</v>
-      </c>
-      <c r="H25" s="4" t="s">
-        <v>190</v>
-      </c>
-      <c r="I25" s="10">
-        <v>4000</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A26" s="10" t="s">
-        <v>103</v>
-      </c>
-      <c r="B26" s="10" t="s">
+      <c r="E26" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F26" t="s">
+        <v>15</v>
+      </c>
+      <c r="G26" s="6">
+        <v>138064624</v>
+      </c>
+      <c r="H26" s="4" t="s">
         <v>192</v>
       </c>
-      <c r="C26" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="D26" s="11">
-        <v>5</v>
-      </c>
-      <c r="E26" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="F26" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="G26" s="12">
-        <v>138064624</v>
-      </c>
-      <c r="H26" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="I26" s="10">
+      <c r="I26">
         <v>4000</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B27" t="s">
         <v>22</v>
@@ -1817,7 +1812,7 @@
         <v>5</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F27" s="1" t="s">
         <v>15</v>
@@ -1826,7 +1821,7 @@
         <v>15640698</v>
       </c>
       <c r="H27" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I27">
         <v>4000</v>
@@ -1834,7 +1829,7 @@
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B28" t="s">
         <v>60</v>
@@ -1846,7 +1841,7 @@
         <v>12</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F28" s="1" t="s">
         <v>15</v>
@@ -1863,7 +1858,7 @@
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B29" t="s">
         <v>64</v>
@@ -1875,7 +1870,7 @@
         <v>3</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F29" s="1" t="s">
         <v>15</v>
@@ -1892,7 +1887,7 @@
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B30" t="s">
         <v>66</v>
@@ -1904,7 +1899,7 @@
         <v>9</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F30" s="1" t="s">
         <v>15</v>
@@ -1921,7 +1916,7 @@
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B31" t="s">
         <v>62</v>
@@ -1933,7 +1928,7 @@
         <v>9</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F31" s="1" t="s">
         <v>15</v>
@@ -1950,7 +1945,7 @@
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B32" t="s">
         <v>30</v>
@@ -1979,7 +1974,7 @@
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B33" t="s">
         <v>32</v>
@@ -2008,7 +2003,7 @@
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B34" t="s">
         <v>35</v>
@@ -2037,7 +2032,7 @@
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B35" t="s">
         <v>37</v>
@@ -2066,7 +2061,7 @@
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B36" t="s">
         <v>39</v>
@@ -2095,7 +2090,7 @@
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B37" t="s">
         <v>41</v>
@@ -2124,7 +2119,7 @@
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B38" t="s">
         <v>50</v>
@@ -2153,7 +2148,7 @@
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B39" t="s">
         <v>70</v>
@@ -2165,7 +2160,7 @@
         <v>4</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F39" s="1" t="s">
         <v>15</v>
@@ -2182,7 +2177,7 @@
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B40" t="s">
         <v>68</v>
@@ -2194,7 +2189,7 @@
         <v>9</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F40" s="1" t="s">
         <v>15</v>
@@ -2211,7 +2206,7 @@
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B41" t="s">
         <v>52</v>
@@ -2223,7 +2218,7 @@
         <v>5</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F41" s="1" t="s">
         <v>15</v>
@@ -2240,7 +2235,7 @@
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B42" s="1" t="s">
         <v>54</v>
@@ -2252,7 +2247,7 @@
         <v>2</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F42" s="1" t="s">
         <v>55</v>
@@ -2269,7 +2264,7 @@
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B43" s="1" t="s">
         <v>57</v>
@@ -2281,7 +2276,7 @@
         <v>6</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F43" s="1" t="s">
         <v>55</v>
@@ -2298,7 +2293,7 @@
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B44" s="1" t="s">
         <v>46</v>
@@ -2327,7 +2322,7 @@
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B45" s="1" t="s">
         <v>47</v>
@@ -2356,7 +2351,7 @@
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B46" s="1" t="s">
         <v>13</v>
@@ -2368,7 +2363,7 @@
         <v>4</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F46" s="1" t="s">
         <v>15</v>
@@ -2385,10 +2380,10 @@
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B47" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C47" s="1" t="s">
         <v>7</v>
@@ -2397,7 +2392,7 @@
         <v>5</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F47" s="1" t="s">
         <v>15</v>
@@ -2413,37 +2408,37 @@
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A48" s="10" t="s">
-        <v>105</v>
-      </c>
-      <c r="B48" s="10" t="s">
-        <v>201</v>
-      </c>
-      <c r="C48" s="11" t="s">
+      <c r="A48" t="s">
+        <v>104</v>
+      </c>
+      <c r="B48" t="s">
+        <v>200</v>
+      </c>
+      <c r="C48" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="D48" s="10">
+      <c r="D48">
         <v>4</v>
       </c>
-      <c r="E48" s="11" t="s">
-        <v>96</v>
-      </c>
-      <c r="F48" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="G48" s="12">
+      <c r="E48" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="F48" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G48" s="6">
         <v>60558384</v>
       </c>
       <c r="H48" s="4" t="s">
-        <v>200</v>
-      </c>
-      <c r="I48" s="10">
+        <v>199</v>
+      </c>
+      <c r="I48">
         <v>3200</v>
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B49" s="1" t="s">
         <v>34</v>
@@ -2472,7 +2467,7 @@
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B50" t="s">
         <v>88</v>
@@ -2501,7 +2496,7 @@
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B51" t="s">
         <v>90</v>
@@ -2513,7 +2508,7 @@
         <v>5</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F51" s="1" t="s">
         <v>15</v>
@@ -2530,10 +2525,10 @@
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B52" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C52" t="s">
         <v>7</v>
@@ -2556,10 +2551,10 @@
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B53" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C53" t="s">
         <v>7</v>
@@ -2568,7 +2563,7 @@
         <v>5</v>
       </c>
       <c r="E53" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F53" t="s">
         <v>15</v>
@@ -2582,10 +2577,10 @@
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B54" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C54" t="s">
         <v>7</v>
@@ -2594,7 +2589,7 @@
         <v>9</v>
       </c>
       <c r="E54" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F54" t="s">
         <v>15</v>
@@ -2608,10 +2603,10 @@
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B55" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C55" t="s">
         <v>7</v>
@@ -2620,7 +2615,7 @@
         <v>5</v>
       </c>
       <c r="E55" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F55" t="s">
         <v>15</v>
@@ -2634,10 +2629,10 @@
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B56" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C56" t="s">
         <v>7</v>
@@ -2646,7 +2641,7 @@
         <v>4</v>
       </c>
       <c r="E56" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F56" t="s">
         <v>15</v>
@@ -2660,10 +2655,10 @@
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B57" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C57" t="s">
         <v>7</v>
@@ -2686,10 +2681,10 @@
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B58" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C58" t="s">
         <v>7</v>
@@ -2712,10 +2707,10 @@
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B59" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C59" s="1" t="s">
         <v>7</v>
@@ -2739,10 +2734,10 @@
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B60" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C60" s="1" t="s">
         <v>7</v>
@@ -2751,7 +2746,7 @@
         <v>9</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F60" s="1" t="s">
         <v>15</v>
@@ -2766,10 +2761,10 @@
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B61" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C61" s="1" t="s">
         <v>7</v>
@@ -2778,7 +2773,7 @@
         <v>5</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F61" s="1" t="s">
         <v>15</v>
@@ -2793,10 +2788,10 @@
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B62" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C62" s="1" t="s">
         <v>7</v>
@@ -2805,7 +2800,7 @@
         <v>9</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F62" s="1" t="s">
         <v>15</v>
@@ -2820,10 +2815,10 @@
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C63" s="1" t="s">
         <v>7</v>
@@ -2847,10 +2842,10 @@
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C64" s="1" t="s">
         <v>7</v>
@@ -2859,7 +2854,7 @@
         <v>9</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F64" s="1" t="s">
         <v>15</v>
@@ -2874,10 +2869,10 @@
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C65" s="1" t="s">
         <v>7</v>
@@ -2886,7 +2881,7 @@
         <v>4</v>
       </c>
       <c r="E65" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F65" s="1" t="s">
         <v>15</v>
@@ -2901,10 +2896,10 @@
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C66" s="1" t="s">
         <v>7</v>
@@ -2913,7 +2908,7 @@
         <v>5</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F66" s="1" t="s">
         <v>15</v>
@@ -2928,10 +2923,10 @@
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C67" s="1" t="s">
         <v>7</v>
@@ -2955,10 +2950,10 @@
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C68" s="1" t="s">
         <v>7</v>
@@ -2982,10 +2977,10 @@
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B69" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C69" t="s">
         <v>7</v>
@@ -2994,7 +2989,7 @@
         <v>5</v>
       </c>
       <c r="E69" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F69" t="s">
         <v>15</v>
@@ -3008,10 +3003,10 @@
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B70" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C70" t="s">
         <v>7</v>
@@ -3034,10 +3029,10 @@
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B71" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C71" t="s">
         <v>7</v>
@@ -3060,10 +3055,10 @@
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B72" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C72" t="s">
         <v>7</v>
@@ -3072,7 +3067,7 @@
         <v>9</v>
       </c>
       <c r="E72" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F72" t="s">
         <v>15</v>
@@ -3086,10 +3081,10 @@
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B73" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C73" t="s">
         <v>7</v>
@@ -3098,7 +3093,7 @@
         <v>5</v>
       </c>
       <c r="E73" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F73" t="s">
         <v>15</v>
@@ -3112,10 +3107,10 @@
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B74" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C74" t="s">
         <v>7</v>
@@ -3138,10 +3133,10 @@
     </row>
     <row r="75" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B75" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C75" t="s">
         <v>7</v>
@@ -3164,10 +3159,10 @@
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B76" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C76" t="s">
         <v>7</v>
@@ -3176,7 +3171,7 @@
         <v>5</v>
       </c>
       <c r="E76" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F76" t="s">
         <v>15</v>
@@ -3190,10 +3185,10 @@
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B77" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C77" t="s">
         <v>7</v>
@@ -3202,7 +3197,7 @@
         <v>9</v>
       </c>
       <c r="E77" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F77" t="s">
         <v>15</v>
@@ -3216,10 +3211,10 @@
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B78" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C78" t="s">
         <v>7</v>
@@ -3242,10 +3237,10 @@
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B79" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C79" t="s">
         <v>7</v>
@@ -3254,7 +3249,7 @@
         <v>4</v>
       </c>
       <c r="E79" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F79" t="s">
         <v>15</v>
@@ -3268,10 +3263,10 @@
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B80" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C80" t="s">
         <v>7</v>
@@ -3294,10 +3289,10 @@
     </row>
     <row r="81" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A81" s="1" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B81" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C81" t="s">
         <v>7</v>
@@ -3306,7 +3301,7 @@
         <v>5</v>
       </c>
       <c r="E81" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F81" t="s">
         <v>15</v>
@@ -3320,10 +3315,10 @@
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
+        <v>146</v>
+      </c>
+      <c r="B82" t="s">
         <v>147</v>
-      </c>
-      <c r="B82" t="s">
-        <v>148</v>
       </c>
       <c r="C82" t="s">
         <v>7</v>
@@ -3332,7 +3327,7 @@
         <v>5</v>
       </c>
       <c r="E82" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F82" t="s">
         <v>15</v>
@@ -3346,10 +3341,10 @@
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B83" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C83" t="s">
         <v>7</v>
@@ -3372,10 +3367,10 @@
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B84" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C84" t="s">
         <v>14</v>
@@ -3384,7 +3379,7 @@
         <v>4</v>
       </c>
       <c r="E84" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F84" t="s">
         <v>15</v>
@@ -3398,10 +3393,10 @@
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B85" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C85" t="s">
         <v>17</v>
@@ -3410,7 +3405,7 @@
         <v>1</v>
       </c>
       <c r="E85" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F85" t="s">
         <v>15</v>
@@ -3424,10 +3419,10 @@
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B86" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C86" t="s">
         <v>7</v>
@@ -3436,10 +3431,10 @@
         <v>3</v>
       </c>
       <c r="E86" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F86" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="G86">
         <v>7560000</v>
@@ -3450,10 +3445,10 @@
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B87" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C87" t="s">
         <v>7</v>
@@ -3476,10 +3471,10 @@
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
+        <v>153</v>
+      </c>
+      <c r="B88" t="s">
         <v>154</v>
-      </c>
-      <c r="B88" t="s">
-        <v>155</v>
       </c>
       <c r="C88" t="s">
         <v>58</v>
@@ -3488,7 +3483,7 @@
         <v>6</v>
       </c>
       <c r="E88" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F88" t="s">
         <v>15</v>
@@ -3502,10 +3497,10 @@
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B89" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C89" t="s">
         <v>58</v>
@@ -3514,7 +3509,7 @@
         <v>2</v>
       </c>
       <c r="E89" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F89" t="s">
         <v>15</v>
@@ -3528,10 +3523,10 @@
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B90" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C90" t="s">
         <v>7</v>
@@ -3540,7 +3535,7 @@
         <v>5</v>
       </c>
       <c r="E90" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F90" t="s">
         <v>15</v>
@@ -3554,10 +3549,10 @@
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B91" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C91" t="s">
         <v>12</v>
@@ -3580,10 +3575,10 @@
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B92" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C92" t="s">
         <v>7</v>
@@ -3592,7 +3587,7 @@
         <v>12</v>
       </c>
       <c r="E92" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F92" t="s">
         <v>15</v>
@@ -3606,10 +3601,10 @@
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B93" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C93" t="s">
         <v>14</v>
@@ -3618,7 +3613,7 @@
         <v>4</v>
       </c>
       <c r="E93" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F93" t="s">
         <v>15</v>
@@ -3632,10 +3627,10 @@
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B94" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C94" t="s">
         <v>7</v>
@@ -3644,7 +3639,7 @@
         <v>9</v>
       </c>
       <c r="E94" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F94" t="s">
         <v>15</v>
@@ -3658,10 +3653,10 @@
     </row>
     <row r="95" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B95" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C95" t="s">
         <v>7</v>
@@ -3670,10 +3665,10 @@
         <v>9</v>
       </c>
       <c r="E95" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F95" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="G95">
         <v>21600000</v>
@@ -3684,10 +3679,10 @@
     </row>
     <row r="96" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B96" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C96" t="s">
         <v>7</v>
@@ -3710,10 +3705,10 @@
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B97" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C97" t="s">
         <v>7</v>
@@ -3736,10 +3731,10 @@
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B98" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C98" t="s">
         <v>7</v>
@@ -3748,7 +3743,7 @@
         <v>3</v>
       </c>
       <c r="E98" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F98" t="s">
         <v>15</v>
@@ -3762,10 +3757,10 @@
     </row>
     <row r="99" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B99" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C99" t="s">
         <v>7</v>
@@ -3774,7 +3769,7 @@
         <v>4</v>
       </c>
       <c r="E99" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F99" t="s">
         <v>15</v>
@@ -3788,10 +3783,10 @@
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B100" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C100" t="s">
         <v>12</v>
@@ -3814,10 +3809,10 @@
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B101" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C101" t="s">
         <v>58</v>
@@ -3826,10 +3821,10 @@
         <v>6</v>
       </c>
       <c r="E101" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F101" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="G101">
         <v>17280000</v>
@@ -3840,10 +3835,10 @@
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B102" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C102" t="s">
         <v>7</v>
@@ -3852,7 +3847,7 @@
         <v>5</v>
       </c>
       <c r="E102" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F102" t="s">
         <v>15</v>
@@ -3866,10 +3861,10 @@
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B103" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C103" t="s">
         <v>7</v>
@@ -3878,10 +3873,10 @@
         <v>5</v>
       </c>
       <c r="E103" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F103" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="G103">
         <v>12000000</v>
@@ -3892,10 +3887,10 @@
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B104" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C104" t="s">
         <v>7</v>
@@ -3918,10 +3913,10 @@
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B105" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C105" t="s">
         <v>7</v>
@@ -3930,7 +3925,7 @@
         <v>9</v>
       </c>
       <c r="E105" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F105" t="s">
         <v>15</v>
@@ -3944,10 +3939,10 @@
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B106" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C106" t="s">
         <v>14</v>
@@ -3956,7 +3951,7 @@
         <v>4</v>
       </c>
       <c r="E106" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F106" t="s">
         <v>15</v>
@@ -3970,10 +3965,10 @@
     </row>
     <row r="107" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B107" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C107" t="s">
         <v>7</v>
@@ -3996,10 +3991,10 @@
     </row>
     <row r="108" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B108" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C108" t="s">
         <v>7</v>
@@ -4008,7 +4003,7 @@
         <v>10</v>
       </c>
       <c r="E108" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F108" t="s">
         <v>15</v>
@@ -4022,10 +4017,10 @@
     </row>
     <row r="109" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B109" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C109" t="s">
         <v>7</v>
@@ -4034,10 +4029,10 @@
         <v>3</v>
       </c>
       <c r="E109" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F109" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="G109">
         <v>7200000</v>
@@ -4048,10 +4043,10 @@
     </row>
     <row r="110" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B110" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C110" t="s">
         <v>12</v>
@@ -4060,7 +4055,7 @@
         <v>9</v>
       </c>
       <c r="E110" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F110" t="s">
         <v>15</v>
@@ -4074,10 +4069,10 @@
     </row>
     <row r="111" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B111" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C111" t="s">
         <v>17</v>

</xml_diff>